<commit_message>
Release 0.1.0: remove list-columns from datasets
washdev and uncnewsletter stored supp_file_type, supp_url,
das_repo_url, and keywords as list-columns, which broke flat-file
exports such as write.csv(). Collapse them into "; "-delimited
character columns in both datasets, update the data dictionary,
documentation, and the data availability article, and regenerate
the extdata exports, README, and pkgdown site.

Document the changes in NEWS.md, bump the version to 0.1.0, and
add alt text to the README word cloud figure.

Closes #8

Assisted-by: Claude claude-fable-5
</commit_message>
<xml_diff>
--- a/inst/extdata/uncnewsletter.xlsx
+++ b/inst/extdata/uncnewsletter.xlsx
@@ -570,7 +570,7 @@
       </c>
       <c r="AB2" t="inlineStr">
         <is>
-          <t>c("drinkingwater", "environmentalpolicy", "healthandsafety")</t>
+          <t>drinkingwater; environmentalpolicy; healthandsafety</t>
         </is>
       </c>
     </row>
@@ -847,7 +847,7 @@
       </c>
       <c r="AB6" t="inlineStr">
         <is>
-          <t>c("Containerbreeding", "Mosquito", "Mosquitolarvae", "Rainwaterharvesting")</t>
+          <t>Containerbreeding; Mosquito; Mosquitolarvae; Rainwaterharvesting</t>
         </is>
       </c>
     </row>
@@ -922,12 +922,12 @@
       </c>
       <c r="Z7" t="inlineStr">
         <is>
-          <t>c("https://deq.nc.gov/about/divisions/mitigation-services/dms-planning/dms-web-map", "https://www.nconemap.gov/", "https://doi.org/10.5066/P96HHBIE", "https://doi.org/10.5066/P9UUT74V", "https://websoilsurvey.nrcs.usda.gov/", "https://doi.org/10.5066/P95PTP5G")</t>
+          <t>https://deq.nc.gov/about/divisions/mitigation-services/dms-planning/dms-web-map; https://www.nconemap.gov/; https://doi.org/10.5066/P96HHBIE; https://doi.org/10.5066/P9UUT74V; https://websoilsurvey.nrcs.usda.gov/; https://doi.org/10.5066/P95PTP5G</t>
         </is>
       </c>
       <c r="AB7" t="inlineStr">
         <is>
-          <t>c("compensatorymitigation", "decisionscience", "knowledgecoproduction", "naturalresourcesmanagement", "research-managementpartnerships", "watershedplanning")</t>
+          <t>compensatorymitigation; decisionscience; knowledgecoproduction; naturalresourcesmanagement; research-managementpartnerships; watershedplanning</t>
         </is>
       </c>
     </row>
@@ -987,7 +987,7 @@
       </c>
       <c r="AB8" t="inlineStr">
         <is>
-          <t>c("Drought", "Communications/decision-making", "Decisionsupport", "Localeffects", "Societalimpacts", "Community")</t>
+          <t>Drought; Communications/decision-making; Decisionsupport; Localeffects; Societalimpacts; Community</t>
         </is>
       </c>
     </row>
@@ -1090,7 +1090,7 @@
       </c>
       <c r="AB9" t="inlineStr">
         <is>
-          <t>c("environmentaljustice", "privatewells", "toxicmetals")</t>
+          <t>environmentaljustice; privatewells; toxicmetals</t>
         </is>
       </c>
     </row>
@@ -1168,7 +1168,7 @@
       </c>
       <c r="AB10" t="inlineStr">
         <is>
-          <t>c("Escherichiacoli", "Plasmid-mediatedquinoloneresistance", "Plasmid-mediatedcolistinresistance", "Poultryworkers", "Chicken", "PoultryEnvironments", "Nigeria")</t>
+          <t>Escherichiacoli; Plasmid-mediatedquinoloneresistance; Plasmid-mediatedcolistinresistance; Poultryworkers; Chicken; PoultryEnvironments; Nigeria</t>
         </is>
       </c>
     </row>
@@ -1236,7 +1236,7 @@
       </c>
       <c r="AB11" t="inlineStr">
         <is>
-          <t>c("Stakeholderanalysis", "FEWS", "Environmentalsustainability", "Transdisciplinaryresearch", "Stakeholderengagement", "Livestockproduction")</t>
+          <t>Stakeholderanalysis; FEWS; Environmentalsustainability; Transdisciplinaryresearch; Stakeholderengagement; Livestockproduction</t>
         </is>
       </c>
     </row>
@@ -1429,7 +1429,7 @@
       </c>
       <c r="AB14" t="inlineStr">
         <is>
-          <t>c("WaterResources", "Life", "EnvironmentalEducation", "Development", "UN2030Agenda")</t>
+          <t>WaterResources; Life; EnvironmentalEducation; Development; UN2030Agenda</t>
         </is>
       </c>
     </row>
@@ -1489,7 +1489,7 @@
       </c>
       <c r="AB15" t="inlineStr">
         <is>
-          <t>c("water", "safedrinkingwateract", "environmentallaw", "law", "policy", "publichealth", "NorthCarolina")</t>
+          <t>water; safedrinkingwateract; environmentallaw; law; policy; publichealth; NorthCarolina</t>
         </is>
       </c>
     </row>
@@ -1632,7 +1632,7 @@
       </c>
       <c r="AB17" t="inlineStr">
         <is>
-          <t>c("Algalblooms", "dynamicalsystems", "mathmodelling", "nutrienttresholdforresolvableblooms")</t>
+          <t>Algalblooms; dynamicalsystems; mathmodelling; nutrienttresholdforresolvableblooms</t>
         </is>
       </c>
     </row>
@@ -1731,7 +1731,7 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>c("xlsx", "docx")</t>
+          <t>xlsx; docx</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
@@ -1800,7 +1800,7 @@
       </c>
       <c r="AB19" t="inlineStr">
         <is>
-          <t>c("autoantibodies", "autoimmune", "crocodilian", "immunetoxicity", "lupus", "onehealth")</t>
+          <t>autoantibodies; autoimmune; crocodilian; immunetoxicity; lupus; onehealth</t>
         </is>
       </c>
     </row>
@@ -2003,7 +2003,7 @@
       </c>
       <c r="AB22" t="inlineStr">
         <is>
-          <t>c("privatewells", "environmentaljustice", "drinkingwater", "testing", "metalcontamination")</t>
+          <t>privatewells; environmentaljustice; drinkingwater; testing; metalcontamination</t>
         </is>
       </c>
     </row>
@@ -2224,7 +2224,7 @@
       </c>
       <c r="AB25" t="inlineStr">
         <is>
-          <t>c("Infrastructure", "NorthCarolina", "Hurricanes", "NaturalDisasters", "PublicOpinion", "WaterSystems")</t>
+          <t>Infrastructure; NorthCarolina; Hurricanes; NaturalDisasters; PublicOpinion; WaterSystems</t>
         </is>
       </c>
     </row>
@@ -2284,7 +2284,7 @@
       </c>
       <c r="AB26" t="inlineStr">
         <is>
-          <t>c("Utilities", "FinancialAssistance", "Durham", "NorthCarolina")</t>
+          <t>Utilities; FinancialAssistance; Durham; NorthCarolina</t>
         </is>
       </c>
     </row>
@@ -2362,7 +2362,7 @@
       </c>
       <c r="AB27" t="inlineStr">
         <is>
-          <t>c("PFAS", "Multimorbidity", "ElectronicHealthRecords", "PFOA", "PFHpA", "Chronicdisease")</t>
+          <t>PFAS; Multimorbidity; ElectronicHealthRecords; PFOA; PFHpA; Chronicdisease</t>
         </is>
       </c>
     </row>
@@ -2450,7 +2450,7 @@
       </c>
       <c r="AB28" t="inlineStr">
         <is>
-          <t>c("DrinkingWater", "Nitrate", "Disinfectionbyproducts", "Trihalomethanes", "Exposureassessment", "Agriculture", "Cohort")</t>
+          <t>DrinkingWater; Nitrate; Disinfectionbyproducts; Trihalomethanes; Exposureassessment; Agriculture; Cohort</t>
         </is>
       </c>
     </row>
@@ -2713,7 +2713,7 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>c("pdf", "xlsx")</t>
+          <t>pdf; xlsx</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
@@ -2791,7 +2791,7 @@
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>c("pdf", "code")</t>
+          <t>pdf; code</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
@@ -2850,7 +2850,7 @@
       </c>
       <c r="AB33" t="inlineStr">
         <is>
-          <t>c("COVID19", "Viralload", "SARSCoV2", "Epidemiology", "Publicandoccupationalhealth", "NorthCarolina", "Diseasesurveillance", "Virustesting")</t>
+          <t>COVID19; Viralload; SARSCoV2; Epidemiology; Publicandoccupationalhealth; NorthCarolina; Diseasesurveillance; Virustesting</t>
         </is>
       </c>
     </row>
@@ -2894,7 +2894,7 @@
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>c("xlsx", "docx")</t>
+          <t>xlsx; docx</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
@@ -3207,7 +3207,7 @@
       </c>
       <c r="AB38" t="inlineStr">
         <is>
-          <t>c("TropicalCyclones", "Spectralwavemodelling", "Coastalhydrodynamics", "Oceancurrents", "Stormsurge", "Barrierislands")</t>
+          <t>TropicalCyclones; Spectralwavemodelling; Coastalhydrodynamics; Oceancurrents; Stormsurge; Barrierislands</t>
         </is>
       </c>
     </row>
@@ -3305,7 +3305,7 @@
       </c>
       <c r="AB39" t="inlineStr">
         <is>
-          <t>c("Pocosin", "Greenhousegases", "Restoration", "Mitigation")</t>
+          <t>Pocosin; Greenhousegases; Restoration; Mitigation</t>
         </is>
       </c>
     </row>
@@ -3385,7 +3385,7 @@
       </c>
       <c r="Z40" t="inlineStr">
         <is>
-          <t>c("https://ameriflux.lbl.gov/sites/siteinfo/US-Cwt", "https://earthengine.google.com", "https://lpdaac.usgs.gov/products/mod16a2gfv006", "https://www.usgs.gov/core-science-systems/nli/landsat/landsat-provisional-actual-evapotranspiration", "https://www.fs.usda.gov/rds/archive/Catalog/RDS-2019-0026", "https://www.fs.usda.gov/rds/archive/catalog/RDS-2013-0013")</t>
+          <t>https://ameriflux.lbl.gov/sites/siteinfo/US-Cwt; https://earthengine.google.com; https://lpdaac.usgs.gov/products/mod16a2gfv006; https://www.usgs.gov/core-science-systems/nli/landsat/landsat-provisional-actual-evapotranspiration; https://www.fs.usda.gov/rds/archive/Catalog/RDS-2019-0026; https://www.fs.usda.gov/rds/archive/catalog/RDS-2013-0013</t>
         </is>
       </c>
       <c r="AA40">
@@ -3393,7 +3393,7 @@
       </c>
       <c r="AB40" t="inlineStr">
         <is>
-          <t>c("Evapotranspiration", "Remotesensing", "Topography", "Forestcomposition", "Landsat", "MODIS")</t>
+          <t>Evapotranspiration; Remotesensing; Topography; Forestcomposition; Landsat; MODIS</t>
         </is>
       </c>
     </row>
@@ -3478,7 +3478,7 @@
       </c>
       <c r="Z41" t="inlineStr">
         <is>
-          <t>c("https://wastewater.covidsurge.mathematica.org", "https://covid19.ncdhhs.gov/dashboard/data-behind-dashboards")</t>
+          <t>https://wastewater.covidsurge.mathematica.org; https://covid19.ncdhhs.gov/dashboard/data-behind-dashboards</t>
         </is>
       </c>
       <c r="AA41">
@@ -3486,7 +3486,7 @@
       </c>
       <c r="AB41" t="inlineStr">
         <is>
-          <t>c("WastewaterMonitoring", "Sars-Covid-2", "Covid-19Surge", "EarlyWarning", "AlertAlgorithm")</t>
+          <t>WastewaterMonitoring; Sars-Covid-2; Covid-19Surge; EarlyWarning; AlertAlgorithm</t>
         </is>
       </c>
     </row>
@@ -3579,7 +3579,7 @@
       </c>
       <c r="AB42" t="inlineStr">
         <is>
-          <t>c("NonmarketEvaluation", "Waterquality", "Urbanstreams", "Statedpreference")</t>
+          <t>NonmarketEvaluation; Waterquality; Urbanstreams; Statedpreference</t>
         </is>
       </c>
     </row>
@@ -3664,7 +3664,7 @@
       </c>
       <c r="Z43" t="inlineStr">
         <is>
-          <t>c("https://scholarworks.iu.edu/dspace/handle/2022/27027", "https://scholarworks.iu.edu/dspace/handle/2022/25638")</t>
+          <t>https://scholarworks.iu.edu/dspace/handle/2022/27027; https://scholarworks.iu.edu/dspace/handle/2022/25638</t>
         </is>
       </c>
       <c r="AA43">
@@ -3672,7 +3672,7 @@
       </c>
       <c r="AB43" t="inlineStr">
         <is>
-          <t>c("Drinkingwater", "Children", "Leadexposure")</t>
+          <t>Drinkingwater; Children; Leadexposure</t>
         </is>
       </c>
     </row>
@@ -3750,7 +3750,7 @@
       </c>
       <c r="AB44" t="inlineStr">
         <is>
-          <t>c("FaecalSludgeTreatment", "Composting", "Temperature-timecritera", "pathogeninactivationmechanism", "compostsanitation")</t>
+          <t>FaecalSludgeTreatment; Composting; Temperature-timecritera; pathogeninactivationmechanism; compostsanitation</t>
         </is>
       </c>
     </row>
@@ -3828,7 +3828,7 @@
       </c>
       <c r="AB45" t="inlineStr">
         <is>
-          <t>c("Hazardmitigation", "compoundevent", "flooding", "ruralresilience", "climatechange")</t>
+          <t>Hazardmitigation; compoundevent; flooding; ruralresilience; climatechange</t>
         </is>
       </c>
     </row>
@@ -3906,7 +3906,7 @@
       </c>
       <c r="AB46" t="inlineStr">
         <is>
-          <t>c("Environmentaljustive", "Ambientwaterquality", "Interfaceswithsociety")</t>
+          <t>Environmentaljustive; Ambientwaterquality; Interfaceswithsociety</t>
         </is>
       </c>
     </row>
@@ -3999,7 +3999,7 @@
       </c>
       <c r="AB47" t="inlineStr">
         <is>
-          <t>c("urban", "nonpointsource", "watershed", "nitrogen", "hydrology", "management")</t>
+          <t>urban; nonpointsource; watershed; nitrogen; hydrology; management</t>
         </is>
       </c>
     </row>
@@ -4092,7 +4092,7 @@
       </c>
       <c r="AB48" t="inlineStr">
         <is>
-          <t>c("sandhills", "seepageflux", "groundwater", "surfacewater", "spatialvariability", "hydrology")</t>
+          <t>sandhills; seepageflux; groundwater; surfacewater; spatialvariability; hydrology</t>
         </is>
       </c>
     </row>
@@ -4177,7 +4177,7 @@
       </c>
       <c r="Z49" t="inlineStr">
         <is>
-          <t>c("https://github.com/bernardoct/WaterPaths/tree/JLWTPAgreementsModel", "https://www.hydroshare.org/resource/3fc8e01960d948a2bd38189dd4e7fa69")</t>
+          <t>https://github.com/bernardoct/WaterPaths/tree/JLWTPAgreementsModel; https://www.hydroshare.org/resource/3fc8e01960d948a2bd38189dd4e7fa69</t>
         </is>
       </c>
       <c r="AA49">
@@ -4185,7 +4185,7 @@
       </c>
       <c r="AB49" t="inlineStr">
         <is>
-          <t>c("waterutility", "cooperation", "demand", "deepuncertainty", "optimization", "financialrisk")</t>
+          <t>waterutility; cooperation; demand; deepuncertainty; optimization; financialrisk</t>
         </is>
       </c>
     </row>
@@ -4270,7 +4270,7 @@
       </c>
       <c r="Z50" t="inlineStr">
         <is>
-          <t>c("https://github.com/acgold/HTF-on-roads", "https://doi.org/10.5281/zenodo.5562568")</t>
+          <t>https://github.com/acgold/HTF-on-roads; https://doi.org/10.5281/zenodo.5562568</t>
         </is>
       </c>
       <c r="AA50">
@@ -4278,7 +4278,7 @@
       </c>
       <c r="AB50" t="inlineStr">
         <is>
-          <t>c("coastaldevelopment", "stormwatermanagement", "infrastructure", "inundationmodeling", "high-tideflooding")</t>
+          <t>coastaldevelopment; stormwatermanagement; infrastructure; inundationmodeling; high-tideflooding</t>
         </is>
       </c>
     </row>
@@ -4366,7 +4366,7 @@
       </c>
       <c r="AB51" t="inlineStr">
         <is>
-          <t>c("erosion", "land-usechange", "legacysediment", "slope-areatreshold", ".", "soilnutrients", "streamchannelinitiation")</t>
+          <t>erosion; land-usechange; legacysediment; slope-areatreshold; .; soilnutrients; streamchannelinitiation</t>
         </is>
       </c>
     </row>
@@ -4434,7 +4434,7 @@
       </c>
       <c r="AB52" t="inlineStr">
         <is>
-          <t>c("collaborativegovernance", "policybeliefs", "regionalwaterplanning", "Gobernanzacolaborativa", "creenciaspolíticas", "planificaciónregionaldelagua", "协作治理", "政策信念", "区域水资源规划")</t>
+          <t>collaborativegovernance; policybeliefs; regionalwaterplanning; Gobernanzacolaborativa; creenciaspolíticas; planificaciónregionaldelagua; 协作治理; 政策信念; 区域水资源规划</t>
         </is>
       </c>
     </row>
@@ -4612,7 +4612,7 @@
       </c>
       <c r="AB54" t="inlineStr">
         <is>
-          <t>c("biology-geologyfeebacks", "DMQ99", "evapotranspiration", "headwaterstreams", "landusechange", "seasonalflashiness", "specificconductance", "streamgauges")</t>
+          <t>biology-geologyfeebacks; DMQ99; evapotranspiration; headwaterstreams; landusechange; seasonalflashiness; specificconductance; streamgauges</t>
         </is>
       </c>
     </row>
@@ -4763,7 +4763,7 @@
       </c>
       <c r="AB56" t="inlineStr">
         <is>
-          <t>c("WASP", "environmentalmodeling", "nanocopper", "nanomaterials", "freswater")</t>
+          <t>WASP; environmentalmodeling; nanocopper; nanomaterials; freswater</t>
         </is>
       </c>
     </row>
@@ -4831,7 +4831,7 @@
       </c>
       <c r="AB57" t="inlineStr">
         <is>
-          <t>c("healtheducation", "healthinformationneeds", "healthprofessionals", "informationdissemination", "informationliteracy", "informationseekingbehavior", "patienteducation", "research", "qualitative")</t>
+          <t>healtheducation; healthinformationneeds; healthprofessionals; informationdissemination; informationliteracy; informationseekingbehavior; patienteducation; research; qualitative</t>
         </is>
       </c>
     </row>
@@ -5002,7 +5002,7 @@
       </c>
       <c r="AB59" t="inlineStr">
         <is>
-          <t>c("crAssphage", "Municipaluntreatedwastewater", "Temporalvariations", "Spatialvariations", "Entericpathogenscorrelations", "Bacteria", "Andviruses", ";", "qPCR", "rt-qPCR")</t>
+          <t>crAssphage; Municipaluntreatedwastewater; Temporalvariations; Spatialvariations; Entericpathogenscorrelations; Bacteria; Andviruses; ;; qPCR; rt-qPCR</t>
         </is>
       </c>
     </row>
@@ -5183,7 +5183,7 @@
       </c>
       <c r="AB61" t="inlineStr">
         <is>
-          <t>c("ArtificialNeuralNetworks", "Geneticprogramming", "Antedcedentenvironmentalconditions", "Temperature", "Salinity", "Oysters")</t>
+          <t>ArtificialNeuralNetworks; Geneticprogramming; Antedcedentenvironmentalconditions; Temperature; Salinity; Oysters</t>
         </is>
       </c>
     </row>
@@ -5336,8 +5336,7 @@
       </c>
       <c r="Z63" t="inlineStr">
         <is>
-          <t>c("https://www.ebi.ac.uk/ena/browser/view/PRJEB40798", "https://www.ebi.ac.uk/ena/browser/view/PRJEB40816", "https://www.ebi.ac.uk/ena/browser/view/PRJEB40815", "https://www.ebi.ac.uk/ena/browser/view/PRJEB27621", "https://www.ebi.ac.uk/ena/browser/view/PRJEB51229", "https://www.ebi.ac.uk/ena/browser/view/ERP015409", "https://bitbucket.org/genomicepidemiology/resfinder_db", "https://ccb-microbe.cs.uni-saarland.de/plsdb/plasmids/download/", "https://www.arb-silva.de/download/arb-files/", "https://benlangmead.github.io/aws-indexes/k2"
-)</t>
+          <t>https://www.ebi.ac.uk/ena/browser/view/PRJEB40798; https://www.ebi.ac.uk/ena/browser/view/PRJEB40816; https://www.ebi.ac.uk/ena/browser/view/PRJEB40815; https://www.ebi.ac.uk/ena/browser/view/PRJEB27621; https://www.ebi.ac.uk/ena/browser/view/PRJEB51229; https://www.ebi.ac.uk/ena/browser/view/ERP015409; https://bitbucket.org/genomicepidemiology/resfinder_db; https://ccb-microbe.cs.uni-saarland.de/plsdb/plasmids/download/; https://www.arb-silva.de/download/arb-files/; https://benlangmead.github.io/aws-indexes/k2</t>
         </is>
       </c>
       <c r="AA63">
@@ -5345,7 +5344,7 @@
       </c>
       <c r="AB63" t="inlineStr">
         <is>
-          <t>c("Antimicrobialresistance", "Metagenomics", "Microbialecology", "Policyandpublichealthinmicrobiology")</t>
+          <t>Antimicrobialresistance; Metagenomics; Microbialecology; Policyandpublichealthinmicrobiology</t>
         </is>
       </c>
     </row>
@@ -5433,7 +5432,7 @@
       </c>
       <c r="AB64" t="inlineStr">
         <is>
-          <t>c("Pretermbirth", "Lowbirthweight", "Adversebirthoutcome", "Pollutedsites", "Superfund", "Industrialsites")</t>
+          <t>Pretermbirth; Lowbirthweight; Adversebirthoutcome; Pollutedsites; Superfund; Industrialsites</t>
         </is>
       </c>
     </row>
@@ -5551,7 +5550,7 @@
       </c>
       <c r="AB65" t="inlineStr">
         <is>
-          <t>c("Carboncycle", "Climate-changemitigation", "Environmentalimpact")</t>
+          <t>Carboncycle; Climate-changemitigation; Environmentalimpact</t>
         </is>
       </c>
     </row>
@@ -5659,7 +5658,7 @@
       </c>
       <c r="AB66" t="inlineStr">
         <is>
-          <t>c("ChemicalEngineering", "Waterresources")</t>
+          <t>ChemicalEngineering; Waterresources</t>
         </is>
       </c>
     </row>
@@ -5745,7 +5744,7 @@
       </c>
       <c r="Z67" t="inlineStr">
         <is>
-          <t>c("https://github.com/TransformingDrainageProject/Drain-Flow-Gap-Filling", "https://github.com/isudatateam/datateam")</t>
+          <t>https://github.com/TransformingDrainageProject/Drain-Flow-Gap-Filling; https://github.com/isudatateam/datateam</t>
         </is>
       </c>
       <c r="AA67">
@@ -5753,7 +5752,7 @@
       </c>
       <c r="AB67" t="inlineStr">
         <is>
-          <t>c("Agriculture", "Environmentalimpact", "Hydrology", "Waterresources")</t>
+          <t>Agriculture; Environmentalimpact; Hydrology; Waterresources</t>
         </is>
       </c>
     </row>
@@ -5978,7 +5977,7 @@
       </c>
       <c r="J70" t="inlineStr">
         <is>
-          <t>c("docx", "tif")</t>
+          <t>docx; tif</t>
         </is>
       </c>
       <c r="K70" t="inlineStr">
@@ -6374,7 +6373,7 @@
       </c>
       <c r="AB74" t="inlineStr">
         <is>
-          <t>c("Cryptosporidium", "Bacillusspores", "MS2coliphage", "bromine", "chlorine", "disinfection", "watertreatment")</t>
+          <t>Cryptosporidium; Bacillusspores; MS2coliphage; bromine; chlorine; disinfection; watertreatment</t>
         </is>
       </c>
     </row>
@@ -6477,7 +6476,7 @@
       </c>
       <c r="AB75" t="inlineStr">
         <is>
-          <t>c("PFASdestruction", "fluoroethers", "GenX", "Nafionbyproduct2", "photolysis")</t>
+          <t>PFASdestruction; fluoroethers; GenX; Nafionbyproduct2; photolysis</t>
         </is>
       </c>
     </row>
@@ -6587,7 +6586,7 @@
       </c>
       <c r="Z76" t="inlineStr">
         <is>
-          <t>c("https://doi.org/10.5281/zenodo.7135955", "https://sunnydayflood.apps.cloudapps.unc.edu", "https://github.com/sunny-day-flooding-project", "https://doi.org/10.5281/zenodo.7017187")</t>
+          <t>https://doi.org/10.5281/zenodo.7135955; https://sunnydayflood.apps.cloudapps.unc.edu; https://github.com/sunny-day-flooding-project; https://doi.org/10.5281/zenodo.7017187</t>
         </is>
       </c>
       <c r="AA76">
@@ -6595,7 +6594,7 @@
       </c>
       <c r="AB76" t="inlineStr">
         <is>
-          <t>c("coastalflooding", "low-costsensors", "hightideflooding", "stormwatermanagement", "coastalinfrastructure", "sealevelrise")</t>
+          <t>coastalflooding; low-costsensors; hightideflooding; stormwatermanagement; coastalinfrastructure; sealevelrise</t>
         </is>
       </c>
     </row>
@@ -6639,7 +6638,7 @@
       </c>
       <c r="J77" t="inlineStr">
         <is>
-          <t>c("docx", "csv")</t>
+          <t>docx; csv</t>
         </is>
       </c>
       <c r="K77" t="inlineStr">
@@ -6712,7 +6711,7 @@
       </c>
       <c r="J78" t="inlineStr">
         <is>
-          <t>c("xlsx", "docx")</t>
+          <t>xlsx; docx</t>
         </is>
       </c>
       <c r="K78" t="inlineStr">
@@ -6761,7 +6760,7 @@
       </c>
       <c r="AB78" t="inlineStr">
         <is>
-          <t>c("PFAS", "Drinkingwater", "USEPA", "PFPrA", "Ultra-shortchain")</t>
+          <t>PFAS; Drinkingwater; USEPA; PFPrA; Ultra-shortchain</t>
         </is>
       </c>
     </row>
@@ -6849,7 +6848,7 @@
       </c>
       <c r="AB79" t="inlineStr">
         <is>
-          <t>c("coastal", "fecalbacteria", "runoff", "stormwater")</t>
+          <t>coastal; fecalbacteria; runoff; stormwater</t>
         </is>
       </c>
     </row>
@@ -6937,7 +6936,7 @@
       </c>
       <c r="AB80" t="inlineStr">
         <is>
-          <t>c("cyanobacteria", "cyanotoxin", "microcystin", "stormwaterpollution", "eutrophication")</t>
+          <t>cyanobacteria; cyanotoxin; microcystin; stormwaterpollution; eutrophication</t>
         </is>
       </c>
     </row>
@@ -7005,7 +7004,7 @@
       </c>
       <c r="AB81" t="inlineStr">
         <is>
-          <t>c("waterscarcity", "waterrecycling", "wastewatertreatmentplants", "nutrients", "phosphorus")</t>
+          <t>waterscarcity; waterrecycling; wastewatertreatmentplants; nutrients; phosphorus</t>
         </is>
       </c>
     </row>
@@ -7118,7 +7117,7 @@
       </c>
       <c r="AB82" t="inlineStr">
         <is>
-          <t>c("HWTS", "POU", "chitosan", "coagulation", "sandfiltration", "bacterialreduction", "virusreduction")</t>
+          <t>HWTS; POU; chitosan; coagulation; sandfiltration; bacterialreduction; virusreduction</t>
         </is>
       </c>
     </row>
@@ -7221,7 +7220,7 @@
       </c>
       <c r="AB83" t="inlineStr">
         <is>
-          <t>c("environmentaljustice", "privatewells", "toxicmetals")</t>
+          <t>environmentaljustice; privatewells; toxicmetals</t>
         </is>
       </c>
     </row>
@@ -7284,7 +7283,7 @@
       </c>
       <c r="AB84" t="inlineStr">
         <is>
-          <t>c("explainability", "LSPmethod", "waterquality", "decision-making")</t>
+          <t>explainability; LSPmethod; waterquality; decision-making</t>
         </is>
       </c>
     </row>
@@ -7369,7 +7368,7 @@
       </c>
       <c r="Z85" t="inlineStr">
         <is>
-          <t>c("https://coast.noaa.gov/slrdata/", "https://coast.noaa.gov/slrdata/", "https://fris.nc.gov/fris/Home.aspx?ST=NC", "https://earthexplorer.usgs.gov/", "https://deq.nc.gov/about/divisions/coastal", "https://www.nconemap.gov/pages/parcels")</t>
+          <t>https://coast.noaa.gov/slrdata/; https://coast.noaa.gov/slrdata/; https://fris.nc.gov/fris/Home.aspx?ST=NC; https://earthexplorer.usgs.gov/; https://deq.nc.gov/about/divisions/coastal; https://www.nconemap.gov/pages/parcels</t>
         </is>
       </c>
       <c r="AA85">
@@ -7377,7 +7376,7 @@
       </c>
       <c r="AB85" t="inlineStr">
         <is>
-          <t>c("wetlands", "nature-basedsolutions", "floodmitigation", "coastalflooding", "tidalwatersheds")</t>
+          <t>wetlands; nature-basedsolutions; floodmitigation; coastalflooding; tidalwatersheds</t>
         </is>
       </c>
     </row>
@@ -7465,7 +7464,7 @@
       </c>
       <c r="AB86" t="inlineStr">
         <is>
-          <t>c("reclaimedwater", "waterreuse", "water-supplysystems", "agro-wastewater", "riskassessment")</t>
+          <t>reclaimedwater; waterreuse; water-supplysystems; agro-wastewater; riskassessment</t>
         </is>
       </c>
     </row>
@@ -7555,7 +7554,7 @@
       </c>
       <c r="Z87" t="inlineStr">
         <is>
-          <t>c("https://www.nconemap.gov/", "https://www.nrcs.usda.gov/wps/portal/nrcs/detail/soils/survey/geo/?cid=nrcs142p2_053628", "https://www.nconemap.gov/", "https://www.nconemap.gov/")</t>
+          <t>https://www.nconemap.gov/; https://www.nrcs.usda.gov/wps/portal/nrcs/detail/soils/survey/geo/?cid=nrcs142p2_053628; https://www.nconemap.gov/; https://www.nconemap.gov/</t>
         </is>
       </c>
       <c r="AA87">
@@ -7563,7 +7562,7 @@
       </c>
       <c r="AB87" t="inlineStr">
         <is>
-          <t>c("geospatialanalysis", "landsuitability", "floodmitigation", "nature-basedsolutions(NBS)", "rurallandscapes", "GeographicInformationSystems(GIS)", "floodresilience")</t>
+          <t>geospatialanalysis; landsuitability; floodmitigation; nature-basedsolutions(NBS); rurallandscapes; GeographicInformationSystems(GIS); floodresilience</t>
         </is>
       </c>
     </row>
@@ -7651,7 +7650,7 @@
       </c>
       <c r="AB88" t="inlineStr">
         <is>
-          <t>c("reclaimedwater", "waterreuse", "water-supplysystems", "agro-wastewater", "riskassessment")</t>
+          <t>reclaimedwater; waterreuse; water-supplysystems; agro-wastewater; riskassessment</t>
         </is>
       </c>
     </row>
@@ -7739,7 +7738,7 @@
       </c>
       <c r="AB89" t="inlineStr">
         <is>
-          <t>c("coastal", "eutrophicationsepticsystems")</t>
+          <t>coastal; eutrophicationsepticsystems</t>
         </is>
       </c>
     </row>
@@ -7802,7 +7801,7 @@
       </c>
       <c r="AB90" t="inlineStr">
         <is>
-          <t>c("hydrologicdrought", "SoutheastUS", "NationalWaterModel")</t>
+          <t>hydrologicdrought; SoutheastUS; NationalWaterModel</t>
         </is>
       </c>
     </row>
@@ -7887,7 +7886,7 @@
       </c>
       <c r="Z91" t="inlineStr">
         <is>
-          <t>c("https://www.census.gov/data/developers/data-sets/acs-5year.html", "https://www.epa.gov/ground-water-and-drinking-water/safe-drinking-water-information-system-sdwis-federal-reporting")</t>
+          <t>https://www.census.gov/data/developers/data-sets/acs-5year.html; https://www.epa.gov/ground-water-and-drinking-water/safe-drinking-water-information-system-sdwis-federal-reporting</t>
         </is>
       </c>
       <c r="AA91">
@@ -7895,7 +7894,7 @@
       </c>
       <c r="AB91" t="inlineStr">
         <is>
-          <t>c("droughtandhealth", "droughtrisk", "LocalMoran", "sI", "droughtvulnerability", "U.S.drought")</t>
+          <t>droughtandhealth; droughtrisk; LocalMoran; sI; droughtvulnerability; U.S.drought</t>
         </is>
       </c>
     </row>
@@ -7973,7 +7972,7 @@
       </c>
       <c r="AB92" t="inlineStr">
         <is>
-          <t>c("environmentalplanning", "policyevaluation", "riparianbuffers")</t>
+          <t>environmentalplanning; policyevaluation; riparianbuffers</t>
         </is>
       </c>
     </row>
@@ -8066,7 +8065,7 @@
       </c>
       <c r="AB93" t="inlineStr">
         <is>
-          <t>c("coastalwetlanddegradation", "remotesensing", "NDVI", "climatechange", "sea-levelrise", "saltwaterintrusion", "hydrologicmodel", "AlligatorRiverNationalWildlifeRefuge", "USA")</t>
+          <t>coastalwetlanddegradation; remotesensing; NDVI; climatechange; sea-levelrise; saltwaterintrusion; hydrologicmodel; AlligatorRiverNationalWildlifeRefuge; USA</t>
         </is>
       </c>
     </row>
@@ -8164,7 +8163,7 @@
       </c>
       <c r="AB94" t="inlineStr">
         <is>
-          <t>c("waterinfrastructure", "waterservices", "waterutilities", "waterbills", "billingfrequency", "customerassistanceprograms(CAPS)", "affordability")</t>
+          <t>waterinfrastructure; waterservices; waterutilities; waterbills; billingfrequency; customerassistanceprograms(CAPS); affordability</t>
         </is>
       </c>
     </row>
@@ -8208,7 +8207,7 @@
       </c>
       <c r="J95" t="inlineStr">
         <is>
-          <t>c("pdf", "xlsx")</t>
+          <t>pdf; xlsx</t>
         </is>
       </c>
       <c r="K95" t="inlineStr">
@@ -8242,7 +8241,7 @@
       </c>
       <c r="AB95" t="inlineStr">
         <is>
-          <t>c("canine", "drinkingwater", "equine", "fluoroether", "OneHealth", "nafionby-product2", "GenXchemicals", "PFOA", "PFOS")</t>
+          <t>canine; drinkingwater; equine; fluoroether; OneHealth; nafionby-product2; GenXchemicals; PFOA; PFOS</t>
         </is>
       </c>
     </row>
@@ -8310,7 +8309,7 @@
       </c>
       <c r="AB96" t="inlineStr">
         <is>
-          <t>c("drinkingwater", "fluoropolymers", "food", "safety", "toxins")</t>
+          <t>drinkingwater; fluoropolymers; food; safety; toxins</t>
         </is>
       </c>
     </row>
@@ -8373,7 +8372,7 @@
       </c>
       <c r="AB97" t="inlineStr">
         <is>
-          <t>c("Airpollution", "Color", "Environmentalpollution", "Environmentalscience", "Impurities")</t>
+          <t>Airpollution; Color; Environmentalpollution; Environmentalscience; Impurities</t>
         </is>
       </c>
     </row>
@@ -8417,7 +8416,7 @@
       </c>
       <c r="J98" t="inlineStr">
         <is>
-          <t>c("pdf", "html")</t>
+          <t>pdf; html</t>
         </is>
       </c>
       <c r="K98" t="inlineStr">
@@ -8466,7 +8465,7 @@
       </c>
       <c r="AB98" t="inlineStr">
         <is>
-          <t>c("lead", "Children", "shealth", "drinkingwater", "machinelearning", "riskassessment")</t>
+          <t>lead; Children; shealth; drinkingwater; machinelearning; riskassessment</t>
         </is>
       </c>
     </row>
@@ -8569,7 +8568,7 @@
       </c>
       <c r="AB99" t="inlineStr">
         <is>
-          <t>c("PFASair-waterinterfacialadsorption", "QSPR", "nonequilibrium", "unsaturatedcolumns", "panfilm")</t>
+          <t>PFASair-waterinterfacialadsorption; QSPR; nonequilibrium; unsaturatedcolumns; panfilm</t>
         </is>
       </c>
     </row>
@@ -8652,7 +8651,7 @@
       </c>
       <c r="AB100" t="inlineStr">
         <is>
-          <t>c("adsorption", "molecules", "nanofibers", "remediation")</t>
+          <t>adsorption; molecules; nanofibers; remediation</t>
         </is>
       </c>
     </row>
@@ -8696,7 +8695,7 @@
       </c>
       <c r="J101" t="inlineStr">
         <is>
-          <t>c("pdf", "xlsx")</t>
+          <t>pdf; xlsx</t>
         </is>
       </c>
       <c r="K101" t="inlineStr">
@@ -8750,7 +8749,7 @@
       </c>
       <c r="AB101" t="inlineStr">
         <is>
-          <t>c("nontargetedanalysis", "anthropogenicchemicals", "wastewater", "landfillleachate", "reverseosmosis")</t>
+          <t>nontargetedanalysis; anthropogenicchemicals; wastewater; landfillleachate; reverseosmosis</t>
         </is>
       </c>
     </row>
@@ -8853,7 +8852,7 @@
       </c>
       <c r="AB102" t="inlineStr">
         <is>
-          <t>c("per-andpolyfluoroalkylsubstances(PFAS)", "presumptivecontamination", "PFAStestingandinvestigation", "AFFF", "PFASwasteanddisposal")</t>
+          <t>per-andpolyfluoroalkylsubstances(PFAS); presumptivecontamination; PFAStestingandinvestigation; AFFF; PFASwasteanddisposal</t>
         </is>
       </c>
     </row>
@@ -8921,7 +8920,7 @@
       </c>
       <c r="AB103" t="inlineStr">
         <is>
-          <t>c("anatomy", "genetics", "infectiousdiseases", "viruses", "wastewater")</t>
+          <t>anatomy; genetics; infectiousdiseases; viruses; wastewater</t>
         </is>
       </c>
     </row>
@@ -9019,7 +9018,7 @@
       </c>
       <c r="AB104" t="inlineStr">
         <is>
-          <t>c("coalash", "lacustrinesediment", "multiproxytracing", "aquaticecosystems")</t>
+          <t>coalash; lacustrinesediment; multiproxytracing; aquaticecosystems</t>
         </is>
       </c>
     </row>
@@ -9087,7 +9086,7 @@
       </c>
       <c r="AB105" t="inlineStr">
         <is>
-          <t>c("waterandsanitationinfrastructure", "disadvantagedunincorporatedcommunities", "environmetaljustice", "participatoryprocess", "sociotechnicaldesign")</t>
+          <t>waterandsanitationinfrastructure; disadvantagedunincorporatedcommunities; environmetaljustice; participatoryprocess; sociotechnicaldesign</t>
         </is>
       </c>
     </row>
@@ -9185,7 +9184,7 @@
       </c>
       <c r="AB106" t="inlineStr">
         <is>
-          <t>c("textiledyes", "environmentalpollution", "cleanwater", "sustainability", "polycarbodiimide", "topologicalpolarsurfacearea(TPSA)", "moleculartransport")</t>
+          <t>textiledyes; environmentalpollution; cleanwater; sustainability; polycarbodiimide; topologicalpolarsurfacearea(TPSA); moleculartransport</t>
         </is>
       </c>
     </row>
@@ -9283,7 +9282,7 @@
       </c>
       <c r="AB107" t="inlineStr">
         <is>
-          <t>c("land-useregression", "molecularmicrobialsourcetracking", "surfacewater", "sediment", "rivernetworks", "animalfeedingoperations", "septicsystems")</t>
+          <t>land-useregression; molecularmicrobialsourcetracking; surfacewater; sediment; rivernetworks; animalfeedingoperations; septicsystems</t>
         </is>
       </c>
     </row>
@@ -9356,7 +9355,7 @@
       </c>
       <c r="AB108" t="inlineStr">
         <is>
-          <t>c("multiplewatersourceuse", "supplementalunimprovedsourceuse", "fecalcontamination", "MonteCarlosimulations", "drinkingwaterquality", "low-andmiddle-incomecountries")</t>
+          <t>multiplewatersourceuse; supplementalunimprovedsourceuse; fecalcontamination; MonteCarlosimulations; drinkingwaterquality; low-andmiddle-incomecountries</t>
         </is>
       </c>
     </row>
@@ -9444,7 +9443,7 @@
       </c>
       <c r="AB109" t="inlineStr">
         <is>
-          <t>c("Microplasticsinrivers", "Watermanagement", "DiversionsAbstraction", "Pairedcatchmentapproach", "Globalmodels")</t>
+          <t>Microplasticsinrivers; Watermanagement; DiversionsAbstraction; Pairedcatchmentapproach; Globalmodels</t>
         </is>
       </c>
     </row>
@@ -9527,7 +9526,7 @@
       </c>
       <c r="AB110" t="inlineStr">
         <is>
-          <t>c("Pocosin", "Carbon", "Methane", "GHG", "Netecosystemexchange", "Hydrologicrestoration", "Peatland", "Evergreenshrubbog", "Watertabledepth", "Eddycovariance", "", "Carbondioxide")</t>
+          <t>Pocosin; Carbon; Methane; GHG; Netecosystemexchange; Hydrologicrestoration; Peatland; Evergreenshrubbog; Watertabledepth; Eddycovariance; Carbondioxide</t>
         </is>
       </c>
     </row>
@@ -9610,7 +9609,7 @@
       </c>
       <c r="AB111" t="inlineStr">
         <is>
-          <t>c("Per-andpolyfluoroalkylsubstances", "PFAS", "Drinkingwater", "Serum", "Humanhealthoutcomes")</t>
+          <t>Per-andpolyfluoroalkylsubstances; PFAS; Drinkingwater; Serum; Humanhealthoutcomes</t>
         </is>
       </c>
     </row>
@@ -9654,7 +9653,7 @@
       </c>
       <c r="J112" t="inlineStr">
         <is>
-          <t>c("pdf", "xlsx")</t>
+          <t>pdf; xlsx</t>
         </is>
       </c>
       <c r="K112" t="inlineStr">
@@ -9695,7 +9694,7 @@
       </c>
       <c r="Z112" t="inlineStr">
         <is>
-          <t>c("https://www.sciencebase.gov/catalog/item/5fad56aad34eb413d5df459c", "https://www.sciencebase.gov/catalog/item/5ab3d60be4b081f61ab5e3d4")</t>
+          <t>https://www.sciencebase.gov/catalog/item/5fad56aad34eb413d5df459c; https://www.sciencebase.gov/catalog/item/5ab3d60be4b081f61ab5e3d4</t>
         </is>
       </c>
       <c r="AA112">
@@ -9703,7 +9702,7 @@
       </c>
       <c r="AB112" t="inlineStr">
         <is>
-          <t>c("Per-andpolyfluoroalkylsubstances", "Drinking-water", "Public-supply", "Private-wellsSources", "Healtheffect")</t>
+          <t>Per-andpolyfluoroalkylsubstances; Drinking-water; Public-supply; Private-wellsSources; Healtheffect</t>
         </is>
       </c>
     </row>
@@ -9811,7 +9810,7 @@
       </c>
       <c r="AB113" t="inlineStr">
         <is>
-          <t>c("Zikavirus", "wastewater-basedepidemiology", "resource-constrainedsettings")</t>
+          <t>Zikavirus; wastewater-basedepidemiology; resource-constrainedsettings</t>
         </is>
       </c>
     </row>
@@ -9914,7 +9913,7 @@
       </c>
       <c r="AB114" t="inlineStr">
         <is>
-          <t>c("Airpollutioncontrol", "Biologicalgastreatment", "Capillaryreactor", "Hydrophobicpollutants", "Segmentedflow")</t>
+          <t>Airpollutioncontrol; Biologicalgastreatment; Capillaryreactor; Hydrophobicpollutants; Segmentedflow</t>
         </is>
       </c>
     </row>
@@ -9997,7 +9996,7 @@
       </c>
       <c r="AB115" t="inlineStr">
         <is>
-          <t>c("Marinemicroalgae", "Dunaliellaviridis", "Flocculation", "Harvesting", "Waterreuse", "Dissolvedorganicmatter")</t>
+          <t>Marinemicroalgae; Dunaliellaviridis; Flocculation; Harvesting; Waterreuse; Dissolvedorganicmatter</t>
         </is>
       </c>
     </row>
@@ -10041,7 +10040,7 @@
       </c>
       <c r="J116" t="inlineStr">
         <is>
-          <t>c("pdf", "xlsx")</t>
+          <t>pdf; xlsx</t>
         </is>
       </c>
       <c r="K116" t="inlineStr">
@@ -10077,7 +10076,7 @@
       </c>
       <c r="Z116" t="inlineStr">
         <is>
-          <t>c("https://www.ncei.noaa.gov", "https://github.com/davidfastovich/gds_climate_reconstruction")</t>
+          <t>https://www.ncei.noaa.gov; https://github.com/davidfastovich/gds_climate_reconstruction</t>
         </is>
       </c>
       <c r="AA116">
@@ -10085,7 +10084,7 @@
       </c>
       <c r="AB116" t="inlineStr">
         <is>
-          <t>c("Palynology", "Plantmacrofossil", "Charcoal", "Paleoclimatereconstruction", "Sea-levelrise", "Wildfire", "Wetlanddevelopment", "Hydroperiod")</t>
+          <t>Palynology; Plantmacrofossil; Charcoal; Paleoclimatereconstruction; Sea-levelrise; Wildfire; Wetlanddevelopment; Hydroperiod</t>
         </is>
       </c>
     </row>
@@ -10158,7 +10157,7 @@
       </c>
       <c r="AB117" t="inlineStr">
         <is>
-          <t>c("Microbiome", "Outdoorair", "Greenspace", "AirborneBacteria", "16SrRNA", "Aerobiome")</t>
+          <t>Microbiome; Outdoorair; Greenspace; AirborneBacteria; 16SrRNA; Aerobiome</t>
         </is>
       </c>
     </row>
@@ -10299,7 +10298,7 @@
       </c>
       <c r="AB119" t="inlineStr">
         <is>
-          <t>c("Watersecurity", "Textanalysis", "Structuraltopicmodeling", "Planning", "Environmentaljustice")</t>
+          <t>Watersecurity; Textanalysis; Structuraltopicmodeling; Planning; Environmentaljustice</t>
         </is>
       </c>
     </row>
@@ -10407,7 +10406,7 @@
       </c>
       <c r="AB120" t="inlineStr">
         <is>
-          <t>c("crAssphage", "Municipaluntreatedwastewater", "Temporalvariations", "Spatialvariations", "Entericpathogenscorrelations", "Bacteria", "Andviruses", "qPCR", "rt-qPCR")</t>
+          <t>crAssphage; Municipaluntreatedwastewater; Temporalvariations; Spatialvariations; Entericpathogenscorrelations; Bacteria; Andviruses; qPCR; rt-qPCR</t>
         </is>
       </c>
     </row>
@@ -10490,7 +10489,7 @@
       </c>
       <c r="AB121" t="inlineStr">
         <is>
-          <t>c("Groundwatercontamination", "Swinelagoons", "Privatewells", "Atmosphericstressors", "Environmentalpollution")</t>
+          <t>Groundwatercontamination; Swinelagoons; Privatewells; Atmosphericstressors; Environmentalpollution</t>
         </is>
       </c>
     </row>
@@ -10573,7 +10572,7 @@
       </c>
       <c r="AB122" t="inlineStr">
         <is>
-          <t>c("Microplastics", "Streamflow", "Urbandevelopment", "Sediment", "Watershed", "Samplingmethod")</t>
+          <t>Microplastics; Streamflow; Urbandevelopment; Sediment; Watershed; Samplingmethod</t>
         </is>
       </c>
     </row>
@@ -10661,7 +10660,7 @@
       </c>
       <c r="AB123" t="inlineStr">
         <is>
-          <t>c("UAV", "UAS", "Rugosity", "Geomorphometry", "Coastalhabitat", "Remotesensing")</t>
+          <t>UAV; UAS; Rugosity; Geomorphometry; Coastalhabitat; Remotesensing</t>
         </is>
       </c>
     </row>
@@ -10705,7 +10704,7 @@
       </c>
       <c r="J124" t="inlineStr">
         <is>
-          <t>c("docx", "pdf")</t>
+          <t>docx; pdf</t>
         </is>
       </c>
       <c r="K124" t="inlineStr">
@@ -10739,7 +10738,7 @@
       </c>
       <c r="AB124" t="inlineStr">
         <is>
-          <t>c("Hospital-aquiredinfection", "Multidrug-resistantpathogen", "Environmentalcleaning", "Probiotic", "Randomized-controlledtrial", "Environmentalhygiene", "MRSAVRE", "Multidrug-resistantGram-negative")</t>
+          <t>Hospital-aquiredinfection; Multidrug-resistantpathogen; Environmentalcleaning; Probiotic; Randomized-controlledtrial; Environmentalhygiene; MRSAVRE; Multidrug-resistantGram-negative</t>
         </is>
       </c>
     </row>
@@ -10817,7 +10816,7 @@
       </c>
       <c r="AB125" t="inlineStr">
         <is>
-          <t>c("Atmosphericforcing", "CapeHatteras", "PEACH", "Atmosphericcyclones", "Atmosphericwarmandcoolseasons")</t>
+          <t>Atmosphericforcing; CapeHatteras; PEACH; Atmosphericcyclones; Atmosphericwarmandcoolseasons</t>
         </is>
       </c>
     </row>
@@ -10910,7 +10909,7 @@
       </c>
       <c r="AB126" t="inlineStr">
         <is>
-          <t>c("Contamination", "Distribution", "Environment", "Healthimpact", "NorthCarolina", "PFASsources")</t>
+          <t>Contamination; Distribution; Environment; Healthimpact; NorthCarolina; PFASsources</t>
         </is>
       </c>
     </row>
@@ -10983,7 +10982,7 @@
       </c>
       <c r="AB127" t="inlineStr">
         <is>
-          <t>c("Landscapechange", "Climatechange", "Attribution", "NeuseRiver", "Sea-levelrise", "Marshloss")</t>
+          <t>Landscapechange; Climatechange; Attribution; NeuseRiver; Sea-levelrise; Marshloss</t>
         </is>
       </c>
     </row>
@@ -11081,7 +11080,7 @@
       </c>
       <c r="AB128" t="inlineStr">
         <is>
-          <t>c("Clustering", "Metals", "Privatewells", "Socialvulnerability", "Geographicdata")</t>
+          <t>Clustering; Metals; Privatewells; Socialvulnerability; Geographicdata</t>
         </is>
       </c>
     </row>
@@ -11164,7 +11163,7 @@
       </c>
       <c r="AB129" t="inlineStr">
         <is>
-          <t>c("Groundwatercontamination", "Swinelagoons", "Privatewells", "Atmosphericstressors", "Environmentalpollution")</t>
+          <t>Groundwatercontamination; Swinelagoons; Privatewells; Atmosphericstressors; Environmentalpollution</t>
         </is>
       </c>
     </row>
@@ -11262,7 +11261,7 @@
       </c>
       <c r="AB130" t="inlineStr">
         <is>
-          <t>c("Microbioreactor", "Volatileorganiccompound", "Biofiltration", "Modeling")</t>
+          <t>Microbioreactor; Volatileorganiccompound; Biofiltration; Modeling</t>
         </is>
       </c>
     </row>
@@ -11370,7 +11369,7 @@
       </c>
       <c r="AB131" t="inlineStr">
         <is>
-          <t>c("Biofiltration", "Cometabolism", "Adsorption", "Emergingcontaminants")</t>
+          <t>Biofiltration; Cometabolism; Adsorption; Emergingcontaminants</t>
         </is>
       </c>
     </row>
@@ -11478,7 +11477,7 @@
       </c>
       <c r="AB132" t="inlineStr">
         <is>
-          <t>c("Subsurfacedrainage", "Subirrigation", "On-farmwaterstorage", "Drainagewaterreuse", "Supplementalirrigation", "Surfacewaterquality")</t>
+          <t>Subsurfacedrainage; Subirrigation; On-farmwaterstorage; Drainagewaterreuse; Supplementalirrigation; Surfacewaterquality</t>
         </is>
       </c>
     </row>
@@ -11639,7 +11638,7 @@
       </c>
       <c r="AB134" t="inlineStr">
         <is>
-          <t>c("Wastewater-basedepidemiology", "Passivesampling", "Mooreswab")</t>
+          <t>Wastewater-basedepidemiology; Passivesampling; Mooreswab</t>
         </is>
       </c>
     </row>
@@ -11722,7 +11721,7 @@
       </c>
       <c r="AB135" t="inlineStr">
         <is>
-          <t>c("Groundwatercontamination", "Swinelagoons", "Privatewells", "Atmosphericstressors", "Environmentalpollution")</t>
+          <t>Groundwatercontamination; Swinelagoons; Privatewells; Atmosphericstressors; Environmentalpollution</t>
         </is>
       </c>
     </row>
@@ -11825,7 +11824,7 @@
       </c>
       <c r="AB136" t="inlineStr">
         <is>
-          <t>c("SARS-CoV-2", "Wastewater-basedepidemiology", "Universitycampus", "Emergingcontaminants", "Disinfectants")</t>
+          <t>SARS-CoV-2; Wastewater-basedepidemiology; Universitycampus; Emergingcontaminants; Disinfectants</t>
         </is>
       </c>
     </row>
@@ -11903,7 +11902,7 @@
       </c>
       <c r="AB137" t="inlineStr">
         <is>
-          <t>c("Geographicinformationsystems", "Ruralgeography", "statisticalanalysis")</t>
+          <t>Geographicinformationsystems; Ruralgeography; statisticalanalysis</t>
         </is>
       </c>
     </row>
@@ -11976,7 +11975,7 @@
       </c>
       <c r="AB138" t="inlineStr">
         <is>
-          <t>c("Forestedwatersheds", "FUTURESmodel", "Landuselandcoverchange(LULCC)", "Hydrologicmodeling", "SoilandWaterAssessmentTool(SWAT)", "Globalclimatemodel")</t>
+          <t>Forestedwatersheds; FUTURESmodel; Landuselandcoverchange(LULCC); Hydrologicmodeling; SoilandWaterAssessmentTool(SWAT); Globalclimatemodel</t>
         </is>
       </c>
     </row>
@@ -12020,7 +12019,7 @@
       </c>
       <c r="J139" t="inlineStr">
         <is>
-          <t>c("xlsx", "docx")</t>
+          <t>xlsx; docx</t>
         </is>
       </c>
       <c r="K139" t="inlineStr">
@@ -12079,7 +12078,7 @@
       </c>
       <c r="AB139" t="inlineStr">
         <is>
-          <t>c("VOC", "Contaminantflux", "Groundwater", "Stream")</t>
+          <t>VOC; Contaminantflux; Groundwater; Stream</t>
         </is>
       </c>
     </row>
@@ -12147,7 +12146,7 @@
       </c>
       <c r="AB140" t="inlineStr">
         <is>
-          <t>c("CoastalaltimetrySealevel", "Waves", "Videocamera", "Tidegauge", "Buoy", "Altimeter", "Significantwaveheight", "Re-trackingalgorithm")</t>
+          <t>CoastalaltimetrySealevel; Waves; Videocamera; Tidegauge; Buoy; Altimeter; Significantwaveheight; Re-trackingalgorithm</t>
         </is>
       </c>
     </row>
@@ -12250,7 +12249,7 @@
       </c>
       <c r="AB141" t="inlineStr">
         <is>
-          <t>c("Wastewater-basedepidemiology", "Sewagesurveillance", "Coronavirus", "COVID", "ddPCR")</t>
+          <t>Wastewater-basedepidemiology; Sewagesurveillance; Coronavirus; COVID; ddPCR</t>
         </is>
       </c>
     </row>
@@ -12348,7 +12347,7 @@
       </c>
       <c r="AB142" t="inlineStr">
         <is>
-          <t>c("Clustering", "Metals", "Privatewells", "Socialvulnerability", "Geographicdata")</t>
+          <t>Clustering; Metals; Privatewells; Socialvulnerability; Geographicdata</t>
         </is>
       </c>
     </row>
@@ -12461,7 +12460,7 @@
       </c>
       <c r="AB143" t="inlineStr">
         <is>
-          <t>c("GHGEmissions", "Waterextractable", "Phosphorus", "Zinc", "Copper", "NorthCarolina")</t>
+          <t>GHGEmissions; Waterextractable; Phosphorus; Zinc; Copper; NorthCarolina</t>
         </is>
       </c>
     </row>
@@ -12534,7 +12533,7 @@
       </c>
       <c r="AB144" t="inlineStr">
         <is>
-          <t>c("Risk", "Compoundhazard", "Flood", "Rural", "Emergencymanagement", "Planning", "CCWE")</t>
+          <t>Risk; Compoundhazard; Flood; Rural; Emergencymanagement; Planning; CCWE</t>
         </is>
       </c>
     </row>
@@ -12637,7 +12636,7 @@
       </c>
       <c r="AB145" t="inlineStr">
         <is>
-          <t>c("ExtraintestinalpathogenicE.coli(ExPEC)", "Foodborneurinarytractinfection(fUTI)", "Concentratedanimalfeedingoperation(CAFO)", "Syndromicsurveillance", "Besag-York-Mollié(BYM)model", "Ecologicalregressionanalysis")</t>
+          <t>ExtraintestinalpathogenicE.coli(ExPEC); Foodborneurinarytractinfection(fUTI); Concentratedanimalfeedingoperation(CAFO); Syndromicsurveillance; Besag-York-Mollié(BYM)model; Ecologicalregressionanalysis</t>
         </is>
       </c>
     </row>
@@ -12720,7 +12719,7 @@
       </c>
       <c r="AB146" t="inlineStr">
         <is>
-          <t>c("Sourceapportionment", "Receptormodels", "PFAS", "Perfluoroalkylsubstances")</t>
+          <t>Sourceapportionment; Receptormodels; PFAS; Perfluoroalkylsubstances</t>
         </is>
       </c>
     </row>
@@ -12808,7 +12807,7 @@
       </c>
       <c r="AB147" t="inlineStr">
         <is>
-          <t>c("Waterquality", "ToxicCyanobacteria", "Airquality", "PM2.5", "Microcystis", "Dolichospermum")</t>
+          <t>Waterquality; ToxicCyanobacteria; Airquality; PM2.5; Microcystis; Dolichospermum</t>
         </is>
       </c>
     </row>
@@ -12916,7 +12915,7 @@
       </c>
       <c r="AB148" t="inlineStr">
         <is>
-          <t>c("Permeance", "Selectivity", "Rejection", "Advectivetransport", "Diffusivetransport")</t>
+          <t>Permeance; Selectivity; Rejection; Advectivetransport; Diffusivetransport</t>
         </is>
       </c>
     </row>
@@ -13014,7 +13013,7 @@
       </c>
       <c r="AB149" t="inlineStr">
         <is>
-          <t>c("Nutrientmanagement", "Livestock", "Agriculture", "Machinelearning", "SatelliteradarSentinel-1")</t>
+          <t>Nutrientmanagement; Livestock; Agriculture; Machinelearning; SatelliteradarSentinel-1</t>
         </is>
       </c>
     </row>
@@ -13058,7 +13057,7 @@
       </c>
       <c r="J150" t="inlineStr">
         <is>
-          <t>c("xlsx", "docx")</t>
+          <t>xlsx; docx</t>
         </is>
       </c>
       <c r="K150" t="inlineStr">
@@ -13102,7 +13101,7 @@
       </c>
       <c r="AB150" t="inlineStr">
         <is>
-          <t>c("Nitrogenremoval", "Denitrification", "Anammox", "nosZ", "hzo", "Sediments")</t>
+          <t>Nitrogenremoval; Denitrification; Anammox; nosZ; hzo; Sediments</t>
         </is>
       </c>
     </row>
@@ -13175,7 +13174,7 @@
       </c>
       <c r="AB151" t="inlineStr">
         <is>
-          <t>c("CAFOs", "Swine", "Hogproduction", "Animalfarming", "Environmentaljustice", "Gastrointestinalillness")</t>
+          <t>CAFOs; Swine; Hogproduction; Animalfarming; Environmentaljustice; Gastrointestinalillness</t>
         </is>
       </c>
     </row>
@@ -13219,7 +13218,7 @@
       </c>
       <c r="J152" t="inlineStr">
         <is>
-          <t>c("xlsx", "docx")</t>
+          <t>xlsx; docx</t>
         </is>
       </c>
       <c r="K152" t="inlineStr">
@@ -13248,7 +13247,7 @@
       </c>
       <c r="AB152" t="inlineStr">
         <is>
-          <t>c("PFAS", "Massload", "Model", "Sourcetracking", "Environmentalmonitoring", "Drinkingwater")</t>
+          <t>PFAS; Massload; Model; Sourcetracking; Environmentalmonitoring; Drinkingwater</t>
         </is>
       </c>
     </row>
@@ -13341,7 +13340,7 @@
       </c>
       <c r="AB153" t="inlineStr">
         <is>
-          <t>c("Animalhusbandry", "Fecalcontamination", "Sanitation", "Hygiene", "Animalfecesmanagement", "Entericpathogens")</t>
+          <t>Animalhusbandry; Fecalcontamination; Sanitation; Hygiene; Animalfecesmanagement; Entericpathogens</t>
         </is>
       </c>
     </row>
@@ -13404,7 +13403,7 @@
       </c>
       <c r="AB154" t="inlineStr">
         <is>
-          <t>c("Naturalinfrastructure", "Wetlandrestoration", "Reforestation", "Watershedmodeling")</t>
+          <t>Naturalinfrastructure; Wetlandrestoration; Reforestation; Watershedmodeling</t>
         </is>
       </c>
     </row>
@@ -13477,7 +13476,7 @@
       </c>
       <c r="AB155" t="inlineStr">
         <is>
-          <t>c("Hydrogeology", "Climatechange", "Sea-levelrise", "Saltwaterintrusion", "Barrier-islandaquifers")</t>
+          <t>Hydrogeology; Climatechange; Sea-levelrise; Saltwaterintrusion; Barrier-islandaquifers</t>
         </is>
       </c>
     </row>
@@ -13555,7 +13554,7 @@
       </c>
       <c r="AB156" t="inlineStr">
         <is>
-          <t>c("Advancedmeteringinfrastructure", "Waterserviceinterruption", "WaterUtilities", "Smartmeters")</t>
+          <t>Advancedmeteringinfrastructure; Waterserviceinterruption; WaterUtilities; Smartmeters</t>
         </is>
       </c>
     </row>
@@ -13653,7 +13652,7 @@
       </c>
       <c r="AB157" t="inlineStr">
         <is>
-          <t>c("Nutrientmanagement", "Livestock", "Agriculture", "Machinelearning", "SatelliteradarSentinel-1")</t>
+          <t>Nutrientmanagement; Livestock; Agriculture; Machinelearning; SatelliteradarSentinel-1</t>
         </is>
       </c>
     </row>
@@ -13746,7 +13745,7 @@
       </c>
       <c r="AB158" t="inlineStr">
         <is>
-          <t>c("Arsenic", "Privatewells", "Watercontamination", "Birthoutcomes", "Epidemiology")</t>
+          <t>Arsenic; Privatewells; Watercontamination; Birthoutcomes; Epidemiology</t>
         </is>
       </c>
     </row>
@@ -13819,7 +13818,7 @@
       </c>
       <c r="AB159" t="inlineStr">
         <is>
-          <t>c("Lanthanumcontainingmaterial", "Lanthanumcarbonate", "Phosphorusremoval", "Wastewatertreatment", "Mineralprecipitation")</t>
+          <t>Lanthanumcontainingmaterial; Lanthanumcarbonate; Phosphorusremoval; Wastewatertreatment; Mineralprecipitation</t>
         </is>
       </c>
     </row>
@@ -13912,7 +13911,7 @@
       </c>
       <c r="AB160" t="inlineStr">
         <is>
-          <t>c("Residencehall", "Asymptomaticsurveillance", "Positivepredictivevalue", "Clinicalcase")</t>
+          <t>Residencehall; Asymptomaticsurveillance; Positivepredictivevalue; Clinicalcase</t>
         </is>
       </c>
     </row>
@@ -14010,7 +14009,7 @@
       </c>
       <c r="AB161" t="inlineStr">
         <is>
-          <t>c("Infiltrationcapacity", "Urbanhydrology", "Urbansoil", "Rainfall-runoffmodels", "Randomforest", "Stormwater")</t>
+          <t>Infiltrationcapacity; Urbanhydrology; Urbansoil; Rainfall-runoffmodels; Randomforest; Stormwater</t>
         </is>
       </c>
     </row>
@@ -14098,7 +14097,7 @@
       </c>
       <c r="AB162" t="inlineStr">
         <is>
-          <t>c("Groundwater", "Microbesampling", "NorthCarolina", "Coliform", "E.coli", "Waterquality")</t>
+          <t>Groundwater; Microbesampling; NorthCarolina; Coliform; E.coli; Waterquality</t>
         </is>
       </c>
     </row>
@@ -14161,7 +14160,7 @@
       </c>
       <c r="AB163" t="inlineStr">
         <is>
-          <t>c("Rurallandscapes", "Nature-basedsolutions", "Costs", "Economics", "Capitalbudgeting", "Floodmitigation")</t>
+          <t>Rurallandscapes; Nature-basedsolutions; Costs; Economics; Capitalbudgeting; Floodmitigation</t>
         </is>
       </c>
     </row>
@@ -14229,7 +14228,7 @@
       </c>
       <c r="AB164" t="inlineStr">
         <is>
-          <t>c("Aquaticecosystems", "Hydrology", "Landuse/landcover", "Physicalhabitat", "Urbanstreams", "Waterquality")</t>
+          <t>Aquaticecosystems; Hydrology; Landuse/landcover; Physicalhabitat; Urbanstreams; Waterquality</t>
         </is>
       </c>
     </row>
@@ -14273,7 +14272,7 @@
       </c>
       <c r="J165" t="inlineStr">
         <is>
-          <t>c("xlsx", "docx")</t>
+          <t>xlsx; docx</t>
         </is>
       </c>
       <c r="K165" t="inlineStr">
@@ -14302,7 +14301,7 @@
       </c>
       <c r="AB165" t="inlineStr">
         <is>
-          <t>c("PFAS", "Massload", "Model", "Sourcetracking", "Environmentalmonitoring", "Drinkingwater")</t>
+          <t>PFAS; Massload; Model; Sourcetracking; Environmentalmonitoring; Drinkingwater</t>
         </is>
       </c>
     </row>
@@ -14395,7 +14394,7 @@
       </c>
       <c r="AB166" t="inlineStr">
         <is>
-          <t>c("SARS-CoV-2", "Wastewater", "COVID-19", "RT-qPCR", "RT-ddPCR", "Wastewater-basedepidemiology(WBE)")</t>
+          <t>SARS-CoV-2; Wastewater; COVID-19; RT-qPCR; RT-ddPCR; Wastewater-basedepidemiology(WBE)</t>
         </is>
       </c>
     </row>
@@ -14478,7 +14477,7 @@
       </c>
       <c r="AB167" t="inlineStr">
         <is>
-          <t>c("Subsurfacedrainage", "Supplementalirrigation", "On-farmwaterstorage", "Irrigationreservoir", "Drainagewaterreuse", "DRAINMOD-DWR")</t>
+          <t>Subsurfacedrainage; Supplementalirrigation; On-farmwaterstorage; Irrigationreservoir; Drainagewaterreuse; DRAINMOD-DWR</t>
         </is>
       </c>
     </row>
@@ -14551,7 +14550,7 @@
       </c>
       <c r="AB168" t="inlineStr">
         <is>
-          <t>c("CAFOs", "Swine", "Hogproduction", "Animalfarming", "Environmentaljustice", "Gastrointestinalillness")</t>
+          <t>CAFOs; Swine; Hogproduction; Animalfarming; Environmentaljustice; Gastrointestinalillness</t>
         </is>
       </c>
     </row>
@@ -14639,7 +14638,7 @@
       </c>
       <c r="AB169" t="inlineStr">
         <is>
-          <t>c("Groundwater", "Microbesampling", "NorthCarolina", "Coliform", "E.coli", "Waterquality")</t>
+          <t>Groundwater; Microbesampling; NorthCarolina; Coliform; E.coli; Waterquality</t>
         </is>
       </c>
     </row>
@@ -14683,7 +14682,7 @@
       </c>
       <c r="J170" t="inlineStr">
         <is>
-          <t>c("xlsx", "docx")</t>
+          <t>xlsx; docx</t>
         </is>
       </c>
       <c r="K170" t="inlineStr">
@@ -14732,7 +14731,7 @@
       </c>
       <c r="AB170" t="inlineStr">
         <is>
-          <t>c("Arsenic", "Manganese", "Lead", "Privatewells", "K-meansclustering", "Geocoding")</t>
+          <t>Arsenic; Manganese; Lead; Privatewells; K-meansclustering; Geocoding</t>
         </is>
       </c>
     </row>
@@ -14805,7 +14804,7 @@
       </c>
       <c r="AB171" t="inlineStr">
         <is>
-          <t>c("Floods", "Hurricanes", "Interruptedtimeseriesanalysis", "Gastrointestinalillness", "Environmentalepidemiology", "Disasterepidemiology")</t>
+          <t>Floods; Hurricanes; Interruptedtimeseriesanalysis; Gastrointestinalillness; Environmentalepidemiology; Disasterepidemiology</t>
         </is>
       </c>
     </row>
@@ -14883,7 +14882,7 @@
       </c>
       <c r="AB172" t="inlineStr">
         <is>
-          <t>c("Bayesiannetworks", "Drinkingwater", "Bloodleadlevels", "Machinelearning", "Riskassessment", "Healthdisparity")</t>
+          <t>Bayesiannetworks; Drinkingwater; Bloodleadlevels; Machinelearning; Riskassessment; Healthdisparity</t>
         </is>
       </c>
     </row>
@@ -14976,7 +14975,7 @@
       </c>
       <c r="AB173" t="inlineStr">
         <is>
-          <t>c("SARS-CoV-2", "Wastewater", "COVID-19", "RT-qPCR", "RT-ddPCR", "Wastewater-basedepidemiology(WBE)")</t>
+          <t>SARS-CoV-2; Wastewater; COVID-19; RT-qPCR; RT-ddPCR; Wastewater-basedepidemiology(WBE)</t>
         </is>
       </c>
     </row>
@@ -15049,7 +15048,7 @@
       </c>
       <c r="AB174" t="inlineStr">
         <is>
-          <t>c("Privatewells", "Householdwatertreatment", "Healthbeliefmodel", "Self-efficacy", "Socialcognitivetheory", "Drinkingwater")</t>
+          <t>Privatewells; Householdwatertreatment; Healthbeliefmodel; Self-efficacy; Socialcognitivetheory; Drinkingwater</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: correct uncnewsletter indexing and country cleaning (#13)
- Manual supplement fix-ups now index uncnewsletter$paperid instead of
  washdev$paperid, so the curated values land on the intended rows
- The correspondence author country is cleaned into its own column
  instead of overwriting first_author_affiliation_country
- Repair Mac Roman bytes in raw washdev.csv cells at read time
  (openxlsx refused to export the invalid UTF-8)
- Regenerate data/*.rda and inst/extdata exports

Closes #13

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/inst/extdata/uncnewsletter.xlsx
+++ b/inst/extdata/uncnewsletter.xlsx
@@ -557,6 +557,11 @@
           <t>North Carolina State University</t>
         </is>
       </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>United States of America</t>
+        </is>
+      </c>
       <c r="Q2" t="inlineStr">
         <is>
           <t>0000-0002-5778-354X</t>
@@ -635,6 +640,11 @@
           <t>North Carolina State University</t>
         </is>
       </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>United States of America</t>
+        </is>
+      </c>
       <c r="W3" t="b">
         <v>0</v>
       </c>
@@ -703,6 +713,11 @@
           <t>University of North Carolina</t>
         </is>
       </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>United States of America</t>
+        </is>
+      </c>
       <c r="Q4" t="inlineStr">
         <is>
           <t>0000-0002-1906-8692</t>
@@ -781,6 +796,11 @@
           <t>Shenyang Ligong University</t>
         </is>
       </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
       <c r="W5" t="b">
         <v>0</v>
       </c>
@@ -839,6 +859,11 @@
           <t>Longwood University</t>
         </is>
       </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>United States of America</t>
+        </is>
+      </c>
       <c r="W6" t="b">
         <v>0</v>
       </c>
@@ -902,6 +927,11 @@
           <t>North Carolina State University</t>
         </is>
       </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>United States of America</t>
+        </is>
+      </c>
       <c r="Q7" t="inlineStr">
         <is>
           <t>0000-0002-2365-6200</t>
@@ -982,6 +1012,11 @@
           <t>University of South Carolina</t>
         </is>
       </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>United States of America</t>
+        </is>
+      </c>
       <c r="W8" t="b">
         <v>0</v>
       </c>
@@ -1064,7 +1099,7 @@
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>United States of America</t>
         </is>
       </c>
       <c r="W9" t="b">
@@ -1145,6 +1180,11 @@
           <t>North Carolina State University</t>
         </is>
       </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>United States of America</t>
+        </is>
+      </c>
       <c r="Q10" t="inlineStr">
         <is>
           <t>0000-0003-4213-6929</t>
@@ -1223,6 +1263,11 @@
           <t>University of Nebraska-Lincoln</t>
         </is>
       </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>United States of America</t>
+        </is>
+      </c>
       <c r="Q11" t="inlineStr">
         <is>
           <t>0000-0002-0371-7125</t>
@@ -1301,6 +1346,11 @@
           <t>University of North Carolina Wilmington</t>
         </is>
       </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>United States of America</t>
+        </is>
+      </c>
       <c r="W12" t="b">
         <v>0</v>
       </c>
@@ -1359,6 +1409,11 @@
           <t>National Renewable Energy Lab NREL</t>
         </is>
       </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>United States of America</t>
+        </is>
+      </c>
       <c r="Q13" t="inlineStr">
         <is>
           <t>0000-0002-3774-9571</t>
@@ -1419,6 +1474,11 @@
           <t>Universidade Regional do Noroeste do Estado do Rio Grande do Sul</t>
         </is>
       </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>Brazil</t>
+        </is>
+      </c>
       <c r="Q14" t="inlineStr">
         <is>
           <t>0000-0003-1591-3622</t>
@@ -1484,6 +1544,11 @@
           <t>Duke Law School</t>
         </is>
       </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>United States of America</t>
+        </is>
+      </c>
       <c r="W15" t="b">
         <v>0</v>
       </c>
@@ -1544,6 +1609,11 @@
           <t>University of North Carolina at Chapel Hill</t>
         </is>
       </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>United States of America</t>
+        </is>
+      </c>
       <c r="Q16" t="inlineStr">
         <is>
           <t>0000-0001-6999-8268</t>
@@ -1624,7 +1694,7 @@
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>United States of America</t>
         </is>
       </c>
       <c r="AA17">
@@ -1687,6 +1757,11 @@
           <t>University of North Carolina</t>
         </is>
       </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>United States of America</t>
+        </is>
+      </c>
       <c r="AA18">
         <v>0</v>
       </c>
@@ -1731,7 +1806,7 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>xlsx; docx</t>
+          <t>xlsx; xlsx; docx</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
@@ -1769,7 +1844,7 @@
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>United States of America</t>
         </is>
       </c>
       <c r="V19" t="inlineStr">
@@ -1855,6 +1930,11 @@
           <t>University of North Carolina</t>
         </is>
       </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>United States of America</t>
+        </is>
+      </c>
       <c r="Q20" t="inlineStr">
         <is>
           <t>0000-0001-8681-0597</t>
@@ -1925,6 +2005,11 @@
           <t>North Carolina State University</t>
         </is>
       </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>United States of America</t>
+        </is>
+      </c>
       <c r="W21" t="b">
         <v>1</v>
       </c>
@@ -1991,6 +2076,11 @@
       <c r="N22" t="inlineStr">
         <is>
           <t>University of North Carolina</t>
+        </is>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>United States of America</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
@@ -2058,6 +2148,11 @@
           <t>University of North Carolina</t>
         </is>
       </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>United States of America</t>
+        </is>
+      </c>
       <c r="Q23" t="inlineStr">
         <is>
           <t>0000-0002-3078-6716</t>
@@ -2146,6 +2241,11 @@
           <t>University of Georgia</t>
         </is>
       </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>United States of America</t>
+        </is>
+      </c>
       <c r="Q24" t="inlineStr">
         <is>
           <t>0000-0003-2112-3846</t>
@@ -2219,6 +2319,11 @@
           <t>Duke University</t>
         </is>
       </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>United States of America</t>
+        </is>
+      </c>
       <c r="W25" t="b">
         <v>0</v>
       </c>
@@ -2279,6 +2384,11 @@
           <t>North Carolina State University</t>
         </is>
       </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>United States of America</t>
+        </is>
+      </c>
       <c r="W26" t="b">
         <v>0</v>
       </c>
@@ -2349,6 +2459,11 @@
           <t>US EPA</t>
         </is>
       </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>United States of America</t>
+        </is>
+      </c>
       <c r="Q27" t="inlineStr">
         <is>
           <t>0000-0002-6322-4349</t>
@@ -2434,7 +2549,7 @@
       </c>
       <c r="T28" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>United States of America</t>
         </is>
       </c>
       <c r="V28" t="inlineStr">
@@ -2537,7 +2652,7 @@
       </c>
       <c r="T29" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>United States of America</t>
         </is>
       </c>
       <c r="W29" t="b">
@@ -2654,6 +2769,11 @@
           <t>University of California</t>
         </is>
       </c>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>United States of America</t>
+        </is>
+      </c>
       <c r="Q31" t="inlineStr">
         <is>
           <t>0000-0002-1050-6721</t>
@@ -2734,6 +2854,11 @@
           <t>WHO</t>
         </is>
       </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
       <c r="W32" t="b">
         <v>1</v>
       </c>
@@ -2834,7 +2959,7 @@
       </c>
       <c r="T33" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>United States of America</t>
         </is>
       </c>
       <c r="V33" t="inlineStr">
@@ -2894,7 +3019,7 @@
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>xlsx; docx</t>
+          <t>xlsx; xlsx; docx</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
@@ -2913,6 +3038,11 @@
       <c r="N34" t="inlineStr">
         <is>
           <t>North Carolina State University</t>
+        </is>
+      </c>
+      <c r="O34" t="inlineStr">
+        <is>
+          <t>United States of America</t>
         </is>
       </c>
       <c r="Q34" t="inlineStr">
@@ -3010,7 +3140,7 @@
       </c>
       <c r="T35" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>United States of America</t>
         </is>
       </c>
       <c r="V35" t="inlineStr">
@@ -3109,6 +3239,11 @@
           <t>independent</t>
         </is>
       </c>
+      <c r="O37" t="inlineStr">
+        <is>
+          <t>United States of America</t>
+        </is>
+      </c>
       <c r="AA37">
         <v>0</v>
       </c>
@@ -3279,7 +3414,7 @@
       </c>
       <c r="T39" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>United States of America</t>
         </is>
       </c>
       <c r="V39" t="inlineStr">
@@ -3370,6 +3505,11 @@
           <t>North Carolina State University</t>
         </is>
       </c>
+      <c r="O40" t="inlineStr">
+        <is>
+          <t>United States of America</t>
+        </is>
+      </c>
       <c r="W40" t="b">
         <v>1</v>
       </c>
@@ -3458,6 +3598,11 @@
           <t>Mathematice Inc.</t>
         </is>
       </c>
+      <c r="O41" t="inlineStr">
+        <is>
+          <t>United States of America</t>
+        </is>
+      </c>
       <c r="Q41" t="inlineStr">
         <is>
           <t>0000-0002-4324-6807</t>
@@ -3551,6 +3696,11 @@
           <t>North Carolina State University</t>
         </is>
       </c>
+      <c r="O42" t="inlineStr">
+        <is>
+          <t>United States of America</t>
+        </is>
+      </c>
       <c r="Q42" t="inlineStr">
         <is>
           <t>0000-0002-5604-8754</t>
@@ -3644,6 +3794,11 @@
           <t>Indiana University</t>
         </is>
       </c>
+      <c r="O43" t="inlineStr">
+        <is>
+          <t>United States of America</t>
+        </is>
+      </c>
       <c r="Q43" t="inlineStr">
         <is>
           <t>0000-0002-5468-0713</t>
@@ -3737,6 +3892,11 @@
           <t>University of North Carolina</t>
         </is>
       </c>
+      <c r="O44" t="inlineStr">
+        <is>
+          <t>United States of America</t>
+        </is>
+      </c>
       <c r="Q44" t="inlineStr">
         <is>
           <t>0000-0002-3317-7318</t>
@@ -3815,6 +3975,11 @@
           <t>East Carolina University</t>
         </is>
       </c>
+      <c r="O45" t="inlineStr">
+        <is>
+          <t>United States of America</t>
+        </is>
+      </c>
       <c r="Q45" t="inlineStr">
         <is>
           <t>0000-0003-2315-7062</t>
@@ -3893,6 +4058,11 @@
           <t>North Carolina State University</t>
         </is>
       </c>
+      <c r="O46" t="inlineStr">
+        <is>
+          <t>United States of America</t>
+        </is>
+      </c>
       <c r="Q46" t="inlineStr">
         <is>
           <t>0000-0003-3160-5363</t>
@@ -3971,6 +4141,11 @@
           <t>University of North Carolina</t>
         </is>
       </c>
+      <c r="O47" t="inlineStr">
+        <is>
+          <t>United States of America</t>
+        </is>
+      </c>
       <c r="Q47" t="inlineStr">
         <is>
           <t>0000-0002-6982-8768</t>
@@ -4043,7 +4218,7 @@
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>misc</t>
+          <t>docx; xlsx; zip; zip; zip</t>
         </is>
       </c>
       <c r="K48" t="inlineStr">
@@ -4062,6 +4237,11 @@
       <c r="N48" t="inlineStr">
         <is>
           <t>University of Utah</t>
+        </is>
+      </c>
+      <c r="O48" t="inlineStr">
+        <is>
+          <t>United States of America</t>
         </is>
       </c>
       <c r="Q48" t="inlineStr">
@@ -4157,6 +4337,11 @@
           <t>University of North Carolina</t>
         </is>
       </c>
+      <c r="O49" t="inlineStr">
+        <is>
+          <t>United States of America</t>
+        </is>
+      </c>
       <c r="Q49" t="inlineStr">
         <is>
           <t>0000-0002-3078-6716</t>
@@ -4250,6 +4435,11 @@
           <t>University of North Carolina</t>
         </is>
       </c>
+      <c r="O50" t="inlineStr">
+        <is>
+          <t>United States of America</t>
+        </is>
+      </c>
       <c r="Q50" t="inlineStr">
         <is>
           <t>0000-0002-0921-0384</t>
@@ -4343,6 +4533,11 @@
           <t>North Carolina State University</t>
         </is>
       </c>
+      <c r="O51" t="inlineStr">
+        <is>
+          <t>United States of America</t>
+        </is>
+      </c>
       <c r="Q51" t="inlineStr">
         <is>
           <t>0000-0001-6115-6322</t>
@@ -4421,6 +4616,11 @@
           <t>University of Georgia</t>
         </is>
       </c>
+      <c r="O52" t="inlineStr">
+        <is>
+          <t>United States of America</t>
+        </is>
+      </c>
       <c r="Q52" t="inlineStr">
         <is>
           <t>0000-0003-2112-3846</t>
@@ -4521,7 +4721,7 @@
       </c>
       <c r="T53" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>United States of America</t>
         </is>
       </c>
       <c r="V53" t="inlineStr">
@@ -4587,6 +4787,11 @@
           <t>Davidson College</t>
         </is>
       </c>
+      <c r="O54" t="inlineStr">
+        <is>
+          <t>United States of America</t>
+        </is>
+      </c>
       <c r="Q54" t="inlineStr">
         <is>
           <t>0000-0002-3799-5019</t>
@@ -4677,6 +4882,11 @@
           <t>Research Triangle Institute</t>
         </is>
       </c>
+      <c r="O55" t="inlineStr">
+        <is>
+          <t>United States of America</t>
+        </is>
+      </c>
       <c r="Q55" t="inlineStr">
         <is>
           <t>0000-0003-3641-737X</t>
@@ -4750,6 +4960,11 @@
           <t>Center for Environmental Measurement &amp; Modeling</t>
         </is>
       </c>
+      <c r="O56" t="inlineStr">
+        <is>
+          <t>United States of America</t>
+        </is>
+      </c>
       <c r="Q56" t="inlineStr">
         <is>
           <t>0000-0001-6231-9437</t>
@@ -4818,6 +5033,11 @@
           <t>North Carolina State University</t>
         </is>
       </c>
+      <c r="O57" t="inlineStr">
+        <is>
+          <t>United States of America</t>
+        </is>
+      </c>
       <c r="Q57" t="inlineStr">
         <is>
           <t>0000-0001-7360-0021</t>
@@ -4886,6 +5106,11 @@
           <t>University of California</t>
         </is>
       </c>
+      <c r="O58" t="inlineStr">
+        <is>
+          <t>United States of America</t>
+        </is>
+      </c>
       <c r="Q58" t="inlineStr">
         <is>
           <t>0000-0002-3039-9927</t>
@@ -4976,7 +5201,7 @@
       </c>
       <c r="T59" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>United States of America</t>
         </is>
       </c>
       <c r="V59" t="inlineStr">
@@ -5074,7 +5299,7 @@
       </c>
       <c r="T60" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>United States of America</t>
         </is>
       </c>
       <c r="V60" t="inlineStr">
@@ -5157,7 +5382,7 @@
       </c>
       <c r="T61" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>United States of America</t>
         </is>
       </c>
       <c r="V61" t="inlineStr">
@@ -5248,6 +5473,11 @@
           <t>North Carolina State University</t>
         </is>
       </c>
+      <c r="O62" t="inlineStr">
+        <is>
+          <t>United States of America</t>
+        </is>
+      </c>
       <c r="W62" t="b">
         <v>0</v>
       </c>
@@ -5295,7 +5525,7 @@
       </c>
       <c r="J63" t="inlineStr">
         <is>
-          <t>pdf</t>
+          <t>pdf; pdf; xlsx; zip; pdf</t>
         </is>
       </c>
       <c r="K63" t="inlineStr">
@@ -5314,6 +5544,11 @@
       <c r="N63" t="inlineStr">
         <is>
           <t>Technical University of Denmark</t>
+        </is>
+      </c>
+      <c r="O63" t="inlineStr">
+        <is>
+          <t>Denmark</t>
         </is>
       </c>
       <c r="Q63" t="inlineStr">
@@ -5409,6 +5644,11 @@
           <t>University of North Carolina</t>
         </is>
       </c>
+      <c r="O64" t="inlineStr">
+        <is>
+          <t>United States of America</t>
+        </is>
+      </c>
       <c r="Q64" t="inlineStr">
         <is>
           <t>0000-0002-3445-6589</t>
@@ -5476,7 +5716,7 @@
       </c>
       <c r="J65" t="inlineStr">
         <is>
-          <t>pdf</t>
+          <t>pdf; pdf; pdf; pdf; xlsx</t>
         </is>
       </c>
       <c r="K65" t="inlineStr">
@@ -5519,7 +5759,7 @@
       </c>
       <c r="T65" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>United States of America</t>
         </is>
       </c>
       <c r="V65" t="inlineStr">
@@ -5632,7 +5872,7 @@
       </c>
       <c r="T66" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>United States of America</t>
         </is>
       </c>
       <c r="V66" t="inlineStr">
@@ -5723,6 +5963,11 @@
           <t>USDA-ARS</t>
         </is>
       </c>
+      <c r="O67" t="inlineStr">
+        <is>
+          <t>United States of America</t>
+        </is>
+      </c>
       <c r="Q67" t="inlineStr">
         <is>
           <t>0000-0002-0176-7815</t>
@@ -5819,7 +6064,7 @@
       </c>
       <c r="O68" t="inlineStr">
         <is>
-          <t>Uganda</t>
+          <t>United States of America</t>
         </is>
       </c>
       <c r="R68" t="inlineStr">
@@ -5884,7 +6129,7 @@
       </c>
       <c r="J69" t="inlineStr">
         <is>
-          <t>pdf</t>
+          <t>pdf; pdf; pdf; pdf</t>
         </is>
       </c>
       <c r="K69" t="inlineStr">
@@ -5922,7 +6167,7 @@
       </c>
       <c r="T69" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>United States of America</t>
         </is>
       </c>
       <c r="V69" t="inlineStr">
@@ -5977,7 +6222,7 @@
       </c>
       <c r="J70" t="inlineStr">
         <is>
-          <t>docx; tif</t>
+          <t>docx; tif; tif; tif</t>
         </is>
       </c>
       <c r="K70" t="inlineStr">
@@ -5996,6 +6241,11 @@
       <c r="N70" t="inlineStr">
         <is>
           <t>Department of Biological &amp; Agricultural Engineering, NC State University, Raleigh, NC, United States of America</t>
+        </is>
+      </c>
+      <c r="O70" t="inlineStr">
+        <is>
+          <t>United States of America</t>
         </is>
       </c>
       <c r="Q70" t="inlineStr">
@@ -6065,7 +6315,7 @@
       </c>
       <c r="J71" t="inlineStr">
         <is>
-          <t>docx</t>
+          <t>docx; docx; docx</t>
         </is>
       </c>
       <c r="K71" t="inlineStr">
@@ -6084,6 +6334,11 @@
       <c r="N71" t="inlineStr">
         <is>
           <t>Nelson Mandela African Institution of Science and Technology, Arusha, Tanzania</t>
+        </is>
+      </c>
+      <c r="O71" t="inlineStr">
+        <is>
+          <t>United Republic of Tanzania</t>
         </is>
       </c>
       <c r="Q71" t="inlineStr">
@@ -6196,7 +6451,7 @@
       </c>
       <c r="T72" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>United States of America</t>
         </is>
       </c>
       <c r="W72" t="b">
@@ -6267,6 +6522,11 @@
           <t>Environmental Intervention Unit, Infectious Disease Division, icddr,b, Dhaka, Bangladesh</t>
         </is>
       </c>
+      <c r="O73" t="inlineStr">
+        <is>
+          <t>Bangladesh</t>
+        </is>
+      </c>
       <c r="Q73" t="inlineStr">
         <is>
           <t>0000-0003-0520-2683</t>
@@ -6362,7 +6622,7 @@
       </c>
       <c r="T74" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>United States of America</t>
         </is>
       </c>
       <c r="W74" t="b">
@@ -6460,7 +6720,7 @@
       </c>
       <c r="T75" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>United States of America</t>
         </is>
       </c>
       <c r="V75" t="inlineStr">
@@ -6563,7 +6823,7 @@
       </c>
       <c r="T76" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>United States of America</t>
         </is>
       </c>
       <c r="V76" t="inlineStr">
@@ -6659,6 +6919,11 @@
           <t>Nicholas Institute for Energy, Environment and Sustainability, Duke University, Durham, North Carolina, United States of America</t>
         </is>
       </c>
+      <c r="O77" t="inlineStr">
+        <is>
+          <t>United States of America</t>
+        </is>
+      </c>
       <c r="Q77" t="inlineStr">
         <is>
           <t>0000-0002-7512-7845</t>
@@ -6732,6 +6997,11 @@
           <t>Natural Resources Defense Council, 111 Sutter St. Floor 20, San Francisco, CA 94104, USA</t>
         </is>
       </c>
+      <c r="O78" t="inlineStr">
+        <is>
+          <t>United States of America</t>
+        </is>
+      </c>
       <c r="R78" t="inlineStr">
         <is>
           <t>Anna Reade</t>
@@ -6825,6 +7095,11 @@
           <t>Department of Health Education and Promotion, East Carolina University, Greenville, NC 27858, USA</t>
         </is>
       </c>
+      <c r="O79" t="inlineStr">
+        <is>
+          <t>United States of America</t>
+        </is>
+      </c>
       <c r="Q79" t="inlineStr">
         <is>
           <t>0000-0003-2664-4763</t>
@@ -6913,6 +7188,11 @@
           <t>Center for Marine Sciences, University of North Carolina Wilmington, 5600 Marvin K. Moss Ln., Wilmington, NC 28409, USA</t>
         </is>
       </c>
+      <c r="O80" t="inlineStr">
+        <is>
+          <t>United States of America</t>
+        </is>
+      </c>
       <c r="Q80" t="inlineStr">
         <is>
           <t>0000-0001-8701-7654</t>
@@ -6991,6 +7271,11 @@
           <t>CIEPQPF, Department of Chemical Engineering, University of Coimbra, 3030-790 Coimbra, Portugal</t>
         </is>
       </c>
+      <c r="O81" t="inlineStr">
+        <is>
+          <t>Portugal</t>
+        </is>
+      </c>
       <c r="Q81" t="inlineStr">
         <is>
           <t>0000-0002-0944-8632</t>
@@ -7091,7 +7376,7 @@
       </c>
       <c r="T82" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>United States of America</t>
         </is>
       </c>
       <c r="V82" t="inlineStr">
@@ -7194,7 +7479,7 @@
       </c>
       <c r="T83" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>United States of America</t>
         </is>
       </c>
       <c r="W83" t="b">
@@ -7275,6 +7560,11 @@
           <t>Department of Computer Science, San Francisco State University, 1600 Holloway Ave, San Francisco, CA 94132, USA</t>
         </is>
       </c>
+      <c r="O84" t="inlineStr">
+        <is>
+          <t>United States of America</t>
+        </is>
+      </c>
       <c r="W84" t="b">
         <v>0</v>
       </c>
@@ -7348,6 +7638,11 @@
           <t>Department of Earth and Ocean Sciences, University of North Carolina Wilmington, 601 S College Rd., Wilmington, NC 28403, USA</t>
         </is>
       </c>
+      <c r="O85" t="inlineStr">
+        <is>
+          <t>United States of America</t>
+        </is>
+      </c>
       <c r="Q85" t="inlineStr">
         <is>
           <t>0000-0002-6591-7237</t>
@@ -7441,6 +7736,11 @@
           <t>Department of Environmental Sciences and Engineering, Gillings School of Global Public Health, The University of North Carolina at Chapel Hill, Chapel Hill, NC 27599, USA</t>
         </is>
       </c>
+      <c r="O86" t="inlineStr">
+        <is>
+          <t>United States of America</t>
+        </is>
+      </c>
       <c r="Q86" t="inlineStr">
         <is>
           <t>0000-0003-1292-0771</t>
@@ -7536,7 +7836,7 @@
       </c>
       <c r="T87" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>United States of America</t>
         </is>
       </c>
       <c r="W87" t="b">
@@ -7627,6 +7927,11 @@
           <t>Department of Environmental Sciences and Engineering, Gillings School of Global Public Health, The University of North Carolina at Chapel Hill, Chapel Hill, NC 27599, USA</t>
         </is>
       </c>
+      <c r="O88" t="inlineStr">
+        <is>
+          <t>United States of America</t>
+        </is>
+      </c>
       <c r="Q88" t="inlineStr">
         <is>
           <t>0000-0003-1292-0771</t>
@@ -7715,6 +8020,11 @@
           <t>Department of Health Education and Promotion, East Carolina University, Greenville, NC 27858, USA</t>
         </is>
       </c>
+      <c r="O89" t="inlineStr">
+        <is>
+          <t>United States of America</t>
+        </is>
+      </c>
       <c r="Q89" t="inlineStr">
         <is>
           <t>0000-0003-2664-4763</t>
@@ -7793,6 +8103,11 @@
           <t>Department of Geosciences, Mississippi State University, Mississippi State, MS 39762, USA</t>
         </is>
       </c>
+      <c r="O90" t="inlineStr">
+        <is>
+          <t>United States of America</t>
+        </is>
+      </c>
       <c r="W90" t="b">
         <v>0</v>
       </c>
@@ -7866,6 +8181,11 @@
           <t>Department of Environmental, Agricultural, and Occupational Health, College of Public Health, University of Nebraska Medical Center, Omaha, NE 68198, USA</t>
         </is>
       </c>
+      <c r="O91" t="inlineStr">
+        <is>
+          <t>United States of America</t>
+        </is>
+      </c>
       <c r="Q91" t="inlineStr">
         <is>
           <t>0000-0003-1143-1191</t>
@@ -7959,6 +8279,11 @@
           <t>Department of City and Regional Planning, University of North Carolina at Chapel Hill, Chapel Hill, NC 27599, USA</t>
         </is>
       </c>
+      <c r="O92" t="inlineStr">
+        <is>
+          <t>United States of America</t>
+        </is>
+      </c>
       <c r="Q92" t="inlineStr">
         <is>
           <t>0000-0002-2834-3764</t>
@@ -8037,6 +8362,11 @@
           <t>Earth and Climate Sciences, Nicholas School of the Environment, Duke University, Durham, NC 27708, USA</t>
         </is>
       </c>
+      <c r="O93" t="inlineStr">
+        <is>
+          <t>United States of America</t>
+        </is>
+      </c>
       <c r="Q93" t="inlineStr">
         <is>
           <t>0000-0001-5793-8583</t>
@@ -8137,7 +8467,7 @@
       </c>
       <c r="T94" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>United States of America</t>
         </is>
       </c>
       <c r="W94" t="b">
@@ -8228,6 +8558,11 @@
           <t>Center for Environmental and Health Effects of PFAS, Department of Biological Sciences, North Carolina State University, Raleigh, North Carolina 27695, United States</t>
         </is>
       </c>
+      <c r="O95" t="inlineStr">
+        <is>
+          <t>United States of America</t>
+        </is>
+      </c>
       <c r="Q95" t="inlineStr">
         <is>
           <t>0000-0003-2954-1110</t>
@@ -8296,6 +8631,11 @@
           <t>Department of Biological Sciences, North Carolina State University, Raleigh, North Carolina 27695, United States</t>
         </is>
       </c>
+      <c r="O96" t="inlineStr">
+        <is>
+          <t>United States of America</t>
+        </is>
+      </c>
       <c r="Q96" t="inlineStr">
         <is>
           <t>0000-0002-5289-1218</t>
@@ -8437,6 +8777,11 @@
           <t>RTI International, Research Triangle Park, North Carolina 27709, United States</t>
         </is>
       </c>
+      <c r="O98" t="inlineStr">
+        <is>
+          <t>United States of America</t>
+        </is>
+      </c>
       <c r="Q98" t="inlineStr">
         <is>
           <t>0000-0001-6293-3672</t>
@@ -8552,7 +8897,7 @@
       </c>
       <c r="T99" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>United States of America</t>
         </is>
       </c>
       <c r="V99" t="inlineStr">
@@ -8640,7 +8985,7 @@
       </c>
       <c r="T100" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>United States of America</t>
         </is>
       </c>
       <c r="W100" t="b">
@@ -8733,7 +9078,7 @@
       </c>
       <c r="T101" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>United States of America</t>
         </is>
       </c>
       <c r="V101" t="inlineStr">
@@ -8836,7 +9181,7 @@
       </c>
       <c r="T102" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>United States of America</t>
         </is>
       </c>
       <c r="V102" t="inlineStr">
@@ -8907,6 +9252,11 @@
           <t>EPCOR Water Services Inc., Edmonton, Alberta T5H 0E8, Canada</t>
         </is>
       </c>
+      <c r="O103" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
       <c r="Q103" t="inlineStr">
         <is>
           <t>0000-0001-9488-8124</t>
@@ -8964,7 +9314,7 @@
       </c>
       <c r="J104" t="inlineStr">
         <is>
-          <t>xlsx</t>
+          <t>xlsx; xlsx; xlsx; xlsx; xlsx; pdf</t>
         </is>
       </c>
       <c r="K104" t="inlineStr">
@@ -9002,7 +9352,7 @@
       </c>
       <c r="T104" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>United States of America</t>
         </is>
       </c>
       <c r="V104" t="inlineStr">
@@ -9073,6 +9423,11 @@
           <t>Department of Anthropology, University of South Florida, Tampa, Florida 33620, United States</t>
         </is>
       </c>
+      <c r="O105" t="inlineStr">
+        <is>
+          <t>United States of America</t>
+        </is>
+      </c>
       <c r="Q105" t="inlineStr">
         <is>
           <t>0000-0003-1966-2680</t>
@@ -9168,7 +9523,7 @@
       </c>
       <c r="T106" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>United States of America</t>
         </is>
       </c>
       <c r="V106" t="inlineStr">
@@ -9271,7 +9626,7 @@
       </c>
       <c r="T107" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>United States of America</t>
         </is>
       </c>
       <c r="W107" t="b">
@@ -9347,6 +9702,11 @@
           <t>Department of Civil, Construction, and Environmental Engineering, North Carolina State University, Fitts-Woolard Hall, 915 Partners Way, Rm 3250, Raleigh, North Carolina 27695, United States</t>
         </is>
       </c>
+      <c r="O108" t="inlineStr">
+        <is>
+          <t>United States of America</t>
+        </is>
+      </c>
       <c r="W108" t="b">
         <v>0</v>
       </c>
@@ -9420,6 +9780,11 @@
           <t>School of Geography, Earth and Environmental Sciences, University of Birmingham, Edgbaston, Birmingham B15 2TT, United Kingdom</t>
         </is>
       </c>
+      <c r="O109" t="inlineStr">
+        <is>
+          <t>United Kingdom of Great Britain and Northern Ireland</t>
+        </is>
+      </c>
       <c r="Q109" t="inlineStr">
         <is>
           <t>0000-0002-7008-0371</t>
@@ -9508,6 +9873,11 @@
           <t>Duke University Wetland Center, Nicholas School of the Environment, Duke University, Box 90333, Durham, NC 27708, USA</t>
         </is>
       </c>
+      <c r="O110" t="inlineStr">
+        <is>
+          <t>United States of America</t>
+        </is>
+      </c>
       <c r="W110" t="b">
         <v>1</v>
       </c>
@@ -9591,6 +9961,11 @@
           <t>Nicholas School of the Environment, Duke University, Durham 27710, NC, USA</t>
         </is>
       </c>
+      <c r="O111" t="inlineStr">
+        <is>
+          <t>United States of America</t>
+        </is>
+      </c>
       <c r="W111" t="b">
         <v>1</v>
       </c>
@@ -9674,6 +10049,11 @@
           <t>U.S. Geological Survey, Lawrenceville, NJ, US</t>
         </is>
       </c>
+      <c r="O112" t="inlineStr">
+        <is>
+          <t>United States of America</t>
+        </is>
+      </c>
       <c r="Q112" t="inlineStr">
         <is>
           <t>0000-0002-1214-4920</t>
@@ -9789,7 +10169,7 @@
       </c>
       <c r="T113" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>United States of America</t>
         </is>
       </c>
       <c r="W113" t="b">
@@ -9978,6 +10358,11 @@
           <t>Department of Civil, Construction, and Environmental Engineering, North Carolina State University, 915 Partners Way, Raleigh, NC 27695, USA</t>
         </is>
       </c>
+      <c r="O115" t="inlineStr">
+        <is>
+          <t>United States of America</t>
+        </is>
+      </c>
       <c r="W115" t="b">
         <v>1</v>
       </c>
@@ -10040,7 +10425,7 @@
       </c>
       <c r="J116" t="inlineStr">
         <is>
-          <t>pdf; xlsx</t>
+          <t>pdf; xlsx; xlsx</t>
         </is>
       </c>
       <c r="K116" t="inlineStr">
@@ -10059,6 +10444,11 @@
       <c r="N116" t="inlineStr">
         <is>
           <t>U.S. Geological Survey, Florence Bascom Geoscience Center, MS 926A, Reston, VA, USA</t>
+        </is>
+      </c>
+      <c r="O116" t="inlineStr">
+        <is>
+          <t>United States of America</t>
         </is>
       </c>
       <c r="W116" t="b">
@@ -10139,6 +10529,11 @@
           <t>United States Environmental Protection Agency, Center for Public Health and Environmental Assessment, Office of Research and Development, Research Triangle Park, NC, USA</t>
         </is>
       </c>
+      <c r="O117" t="inlineStr">
+        <is>
+          <t>United States of America</t>
+        </is>
+      </c>
       <c r="W117" t="b">
         <v>1</v>
       </c>
@@ -10222,6 +10617,11 @@
           <t>Department of Environmental Sciences and Engineering, Gillings School of Global Public Health, University of North Carolina at Chapel Hill, Chapel Hill, NC, USA</t>
         </is>
       </c>
+      <c r="O118" t="inlineStr">
+        <is>
+          <t>United States of America</t>
+        </is>
+      </c>
       <c r="W118" t="b">
         <v>0</v>
       </c>
@@ -10280,6 +10680,11 @@
           <t>The Roux Institute, Northeastern University 100 Fore St. Portland, ME USA 04101</t>
         </is>
       </c>
+      <c r="O119" t="inlineStr">
+        <is>
+          <t>United States of America</t>
+        </is>
+      </c>
       <c r="W119" t="b">
         <v>1</v>
       </c>
@@ -10385,7 +10790,7 @@
       </c>
       <c r="T120" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>United States of America</t>
         </is>
       </c>
       <c r="W120" t="b">
@@ -10471,6 +10876,11 @@
           <t>Haub School of Environment and Natural Resources, University of Wyoming, USA</t>
         </is>
       </c>
+      <c r="O121" t="inlineStr">
+        <is>
+          <t>United States of America</t>
+        </is>
+      </c>
       <c r="W121" t="b">
         <v>1</v>
       </c>
@@ -10554,6 +10964,11 @@
           <t>Biological and Agricultural Engineering, North Carolina State University, Raleigh, NC, USA</t>
         </is>
       </c>
+      <c r="O122" t="inlineStr">
+        <is>
+          <t>United States of America</t>
+        </is>
+      </c>
       <c r="W122" t="b">
         <v>1</v>
       </c>
@@ -10637,6 +11052,11 @@
           <t>School of Forest, Fisheries, and Geomatics Sciences, University of Florida, Gainesville, FL, USA</t>
         </is>
       </c>
+      <c r="O123" t="inlineStr">
+        <is>
+          <t>United States of America</t>
+        </is>
+      </c>
       <c r="Q123" t="inlineStr">
         <is>
           <t>0000-0002-2843-4965</t>
@@ -10725,6 +11145,11 @@
           <t>Institute of Hygiene and Environmental Medicine, Charité–Universitätsmedizin Berlin, Corporate Member of Freie Universität Berlin, Humboldt-Universität zu Berlin and Berlin Institute of Health, Berlin, Germany</t>
         </is>
       </c>
+      <c r="O124" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
       <c r="Q124" t="inlineStr">
         <is>
           <t>0000-0002-1225-9023</t>
@@ -10793,6 +11218,11 @@
           <t>University of North Carolina, Chapel Hill, NC, USA</t>
         </is>
       </c>
+      <c r="O125" t="inlineStr">
+        <is>
+          <t>United States of America</t>
+        </is>
+      </c>
       <c r="Q125" t="inlineStr">
         <is>
           <t>0000-0001-6309-1403</t>
@@ -10873,7 +11303,7 @@
       </c>
       <c r="O126" t="inlineStr">
         <is>
-          <t>United States of America</t>
+          <t>Bangladesh</t>
         </is>
       </c>
       <c r="R126" t="inlineStr">
@@ -10888,7 +11318,7 @@
       </c>
       <c r="T126" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>United States of America</t>
         </is>
       </c>
       <c r="W126" t="b">
@@ -10964,6 +11394,11 @@
           <t>Earth Surface Systems Program, University of Kentucky, USA</t>
         </is>
       </c>
+      <c r="O127" t="inlineStr">
+        <is>
+          <t>United States of America</t>
+        </is>
+      </c>
       <c r="W127" t="b">
         <v>1</v>
       </c>
@@ -11054,7 +11489,7 @@
       </c>
       <c r="T128" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>United States of America</t>
         </is>
       </c>
       <c r="W128" t="b">
@@ -11145,6 +11580,11 @@
           <t>Haub School of Environment and Natural Resources, University of Wyoming, USA</t>
         </is>
       </c>
+      <c r="O129" t="inlineStr">
+        <is>
+          <t>United States of America</t>
+        </is>
+      </c>
       <c r="W129" t="b">
         <v>1</v>
       </c>
@@ -11235,7 +11675,7 @@
       </c>
       <c r="T130" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>United States of America</t>
         </is>
       </c>
       <c r="V130" t="inlineStr">
@@ -11343,7 +11783,7 @@
       </c>
       <c r="T131" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>United States of America</t>
         </is>
       </c>
       <c r="V131" t="inlineStr">
@@ -11456,7 +11896,7 @@
       </c>
       <c r="T132" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>United States of America</t>
         </is>
       </c>
       <c r="W132" t="b">
@@ -11532,6 +11972,11 @@
           <t>University of North Carolina at Chapel Hill, Institute of Marine Sciences, Morehead City NC 28557, USA</t>
         </is>
       </c>
+      <c r="O133" t="inlineStr">
+        <is>
+          <t>United States of America</t>
+        </is>
+      </c>
       <c r="W133" t="b">
         <v>0</v>
       </c>
@@ -11617,7 +12062,7 @@
       </c>
       <c r="T134" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>United States of America</t>
         </is>
       </c>
       <c r="W134" t="b">
@@ -11703,6 +12148,11 @@
           <t>Haub School of Environment and Natural Resources, University of Wyoming, USA</t>
         </is>
       </c>
+      <c r="O135" t="inlineStr">
+        <is>
+          <t>United States of America</t>
+        </is>
+      </c>
       <c r="W135" t="b">
         <v>1</v>
       </c>
@@ -11879,6 +12329,11 @@
           <t>North Carolina Central University, Department of Environmental, Earth and Geospatial Sciences, 1246 Mary M, Townes Science Complex, 1801 Fayetteville St., Durham, NC, 27707, USA</t>
         </is>
       </c>
+      <c r="O137" t="inlineStr">
+        <is>
+          <t>United States of America</t>
+        </is>
+      </c>
       <c r="Q137" t="inlineStr">
         <is>
           <t>0000-0001-9333-9641</t>
@@ -11957,6 +12412,11 @@
           <t>North Carolina State University, Department of Forestry and Environmental Resources, 2800 Faucette Dr, Raleigh, NC 27695, USA</t>
         </is>
       </c>
+      <c r="O138" t="inlineStr">
+        <is>
+          <t>United States of America</t>
+        </is>
+      </c>
       <c r="W138" t="b">
         <v>1</v>
       </c>
@@ -12057,7 +12517,7 @@
       </c>
       <c r="T139" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>United States of America</t>
         </is>
       </c>
       <c r="W139" t="b">
@@ -12133,6 +12593,11 @@
           <t>Ecosystems and Fishery Resources Laboratory, Institute of Fisheries and Aquatic Sciences, University of Douala, BP 2701 Douala, Cameroon</t>
         </is>
       </c>
+      <c r="O140" t="inlineStr">
+        <is>
+          <t>Cameroon</t>
+        </is>
+      </c>
       <c r="Q140" t="inlineStr">
         <is>
           <t>0000-0001-7724-5805</t>
@@ -12228,7 +12693,7 @@
       </c>
       <c r="T141" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>United States of America</t>
         </is>
       </c>
       <c r="W141" t="b">
@@ -12321,7 +12786,7 @@
       </c>
       <c r="T142" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>United States of America</t>
         </is>
       </c>
       <c r="W142" t="b">
@@ -12434,7 +12899,7 @@
       </c>
       <c r="T143" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>United States of America</t>
         </is>
       </c>
       <c r="V143" t="inlineStr">
@@ -12515,6 +12980,11 @@
           <t>Dr. John Lining Professor of Physics and Director of the James B. Near Center for Climate Studies, The Citadel, 171 Moultrie Street, Charleston, SC, USA</t>
         </is>
       </c>
+      <c r="O144" t="inlineStr">
+        <is>
+          <t>United States of America</t>
+        </is>
+      </c>
       <c r="W144" t="b">
         <v>1</v>
       </c>
@@ -12615,7 +13085,7 @@
       </c>
       <c r="T145" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>United States of America</t>
         </is>
       </c>
       <c r="W145" t="b">
@@ -12676,11 +13146,11 @@
         <v>1</v>
       </c>
       <c r="I146">
-        <v>13</v>
+        <v>2</v>
       </c>
       <c r="J146" t="inlineStr">
         <is>
-          <t>misc</t>
+          <t>docx; zip</t>
         </is>
       </c>
       <c r="K146" t="inlineStr">
@@ -12699,6 +13169,11 @@
       <c r="N146" t="inlineStr">
         <is>
           <t>Department of Biological Sciences, North Carolina State University, Raleigh, NC, USA</t>
+        </is>
+      </c>
+      <c r="O146" t="inlineStr">
+        <is>
+          <t>United States of America</t>
         </is>
       </c>
       <c r="W146" t="b">
@@ -12784,6 +13259,11 @@
           <t>UNC-Chapel Hill, Earth, Marine, and Environmental Sciences, Institute of Marine Sciences, 3431 Arendell St., Morehead City, NC 28577, United States of America</t>
         </is>
       </c>
+      <c r="O147" t="inlineStr">
+        <is>
+          <t>United States of America</t>
+        </is>
+      </c>
       <c r="Q147" t="inlineStr">
         <is>
           <t>0000-0001-8823-0457</t>
@@ -12889,7 +13369,7 @@
       </c>
       <c r="T148" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>United States of America</t>
         </is>
       </c>
       <c r="V148" t="inlineStr">
@@ -12997,7 +13477,7 @@
       </c>
       <c r="T149" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>United States of America</t>
         </is>
       </c>
       <c r="V149" t="inlineStr">
@@ -13057,7 +13537,7 @@
       </c>
       <c r="J150" t="inlineStr">
         <is>
-          <t>xlsx; docx</t>
+          <t>xlsx; xlsx; xlsx; xlsx; xlsx; xlsx; xlsx; xlsx; xlsx; xlsx; docx; docx</t>
         </is>
       </c>
       <c r="K150" t="inlineStr">
@@ -13076,6 +13556,11 @@
       <c r="N150" t="inlineStr">
         <is>
           <t>Department of Biological Sciences, Virginia Institute of Marine Science, William &amp; Mary, Gloucester Point, VA, USA</t>
+        </is>
+      </c>
+      <c r="O150" t="inlineStr">
+        <is>
+          <t>United States of America</t>
         </is>
       </c>
       <c r="Q150" t="inlineStr">
@@ -13166,6 +13651,11 @@
           <t>Department of Epidemiology, Gillings School of Global Public Health, University of North Carolina, Chapel Hill, NC 27599, USA</t>
         </is>
       </c>
+      <c r="O151" t="inlineStr">
+        <is>
+          <t>United States of America</t>
+        </is>
+      </c>
       <c r="W151" t="b">
         <v>0</v>
       </c>
@@ -13218,7 +13708,7 @@
       </c>
       <c r="J152" t="inlineStr">
         <is>
-          <t>xlsx; docx</t>
+          <t>xlsx; xlsx; docx</t>
         </is>
       </c>
       <c r="K152" t="inlineStr">
@@ -13237,6 +13727,11 @@
       <c r="N152" t="inlineStr">
         <is>
           <t>Department of Marine, Earth, and Atmospheric Sciences, North Carolina State University, Raleigh, NC, United States</t>
+        </is>
+      </c>
+      <c r="O152" t="inlineStr">
+        <is>
+          <t>United States of America</t>
         </is>
       </c>
       <c r="W152" t="b">
@@ -13287,11 +13782,11 @@
         <v>1</v>
       </c>
       <c r="I153">
-        <v>13</v>
+        <v>2</v>
       </c>
       <c r="J153" t="inlineStr">
         <is>
-          <t>misc</t>
+          <t>pdf; docx</t>
         </is>
       </c>
       <c r="K153" t="inlineStr">
@@ -13329,7 +13824,7 @@
       </c>
       <c r="T153" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>United States of America</t>
         </is>
       </c>
       <c r="W153" t="b">
@@ -13395,6 +13890,11 @@
           <t>Department of Biological and Agricultural Engineering, North Carolina State University, 3100 Faucette Dr., Raleigh, NC 27695, United States of America</t>
         </is>
       </c>
+      <c r="O154" t="inlineStr">
+        <is>
+          <t>United States of America</t>
+        </is>
+      </c>
       <c r="W154" t="b">
         <v>0</v>
       </c>
@@ -13458,6 +13958,11 @@
           <t>School for Environment and Sustainability, University of Michigan, MI, 48109, Ann Arbor, USA</t>
         </is>
       </c>
+      <c r="O155" t="inlineStr">
+        <is>
+          <t>United States of America</t>
+        </is>
+      </c>
       <c r="W155" t="b">
         <v>1</v>
       </c>
@@ -13531,6 +14036,11 @@
           <t>North Carolina State University, Department of Civil, Construction and Environmental Engineering Raleigh, NC, USA</t>
         </is>
       </c>
+      <c r="O156" t="inlineStr">
+        <is>
+          <t>United States of America</t>
+        </is>
+      </c>
       <c r="Q156" t="inlineStr">
         <is>
           <t>0000-0003-1322-1948</t>
@@ -13636,7 +14146,7 @@
       </c>
       <c r="T157" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>United States of America</t>
         </is>
       </c>
       <c r="V157" t="inlineStr">
@@ -13734,7 +14244,7 @@
       </c>
       <c r="T158" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>United States of America</t>
         </is>
       </c>
       <c r="W158" t="b">
@@ -13810,6 +14320,11 @@
           <t>Key Laboratory of Eco-environments in Three Gorges Reservoir Region, Ministry of Education, College of Environment and Ecology, Chongqing University, Chongqing 400044, China</t>
         </is>
       </c>
+      <c r="O159" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
       <c r="W159" t="b">
         <v>0</v>
       </c>
@@ -13900,7 +14415,7 @@
       </c>
       <c r="T160" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>United States of America</t>
         </is>
       </c>
       <c r="W160" t="b">
@@ -13993,7 +14508,7 @@
       </c>
       <c r="T161" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>United States of America</t>
         </is>
       </c>
       <c r="V161" t="inlineStr">
@@ -14081,7 +14596,7 @@
       </c>
       <c r="T162" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>United States of America</t>
         </is>
       </c>
       <c r="V162" t="inlineStr">
@@ -14152,6 +14667,11 @@
           <t>Department of Forestry and Environmental Resources, North Carolina State University, Raleigh, N.C., U.SA.</t>
         </is>
       </c>
+      <c r="O163" t="inlineStr">
+        <is>
+          <t>United States of America</t>
+        </is>
+      </c>
       <c r="W163" t="b">
         <v>0</v>
       </c>
@@ -14215,6 +14735,11 @@
           <t>University of North Carolina at Greensboro, Department of Geography, Environment, and Sustainability, 237 Graham Bldg., PO Box 26170, Greensboro, NC, 27402-6170, USA</t>
         </is>
       </c>
+      <c r="O164" t="inlineStr">
+        <is>
+          <t>United States of America</t>
+        </is>
+      </c>
       <c r="Q164" t="inlineStr">
         <is>
           <t>0000-0002-9380-7625</t>
@@ -14272,7 +14797,7 @@
       </c>
       <c r="J165" t="inlineStr">
         <is>
-          <t>xlsx; docx</t>
+          <t>xlsx; xlsx; docx</t>
         </is>
       </c>
       <c r="K165" t="inlineStr">
@@ -14291,6 +14816,11 @@
       <c r="N165" t="inlineStr">
         <is>
           <t>Department of Marine, Earth, and Atmospheric Sciences, North Carolina State University, Raleigh, NC, United States</t>
+        </is>
+      </c>
+      <c r="O165" t="inlineStr">
+        <is>
+          <t>United States of America</t>
         </is>
       </c>
       <c r="W165" t="b">
@@ -14383,7 +14913,7 @@
       </c>
       <c r="T166" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>United States of America</t>
         </is>
       </c>
       <c r="W166" t="b">
@@ -14466,7 +14996,7 @@
       </c>
       <c r="T167" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>United States of America</t>
         </is>
       </c>
       <c r="W167" t="b">
@@ -14542,6 +15072,11 @@
           <t>Department of Epidemiology, Gillings School of Global Public Health, University of North Carolina, Chapel Hill, NC 27599, USA</t>
         </is>
       </c>
+      <c r="O168" t="inlineStr">
+        <is>
+          <t>United States of America</t>
+        </is>
+      </c>
       <c r="W168" t="b">
         <v>0</v>
       </c>
@@ -14622,7 +15157,7 @@
       </c>
       <c r="T169" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>United States of America</t>
         </is>
       </c>
       <c r="V169" t="inlineStr">
@@ -14682,7 +15217,7 @@
       </c>
       <c r="J170" t="inlineStr">
         <is>
-          <t>xlsx; docx</t>
+          <t>xlsx; docx; docx</t>
         </is>
       </c>
       <c r="K170" t="inlineStr">
@@ -14720,7 +15255,7 @@
       </c>
       <c r="T170" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>United States of America</t>
         </is>
       </c>
       <c r="W170" t="b">
@@ -14796,6 +15331,11 @@
           <t>Department of Epidemiology, Gillings School of Global Public Health, University of North Carolina, Chapel Hill, NC 27599, USA</t>
         </is>
       </c>
+      <c r="O171" t="inlineStr">
+        <is>
+          <t>United States of America</t>
+        </is>
+      </c>
       <c r="W171" t="b">
         <v>0</v>
       </c>
@@ -14869,6 +15409,11 @@
           <t>Department of Environmental Sciences and Engineering, Gillings School of Global Public Health, University of North Carolina at Chapel Hill, 135 Dauer Drive, Chapel Hill, NC, 27599, USA</t>
         </is>
       </c>
+      <c r="O172" t="inlineStr">
+        <is>
+          <t>United States of America</t>
+        </is>
+      </c>
       <c r="Q172" t="inlineStr">
         <is>
           <t>0000-0001-6293-3672</t>
@@ -14964,7 +15509,7 @@
       </c>
       <c r="T173" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>United States of America</t>
         </is>
       </c>
       <c r="W173" t="b">
@@ -15038,6 +15583,11 @@
       <c r="N174" t="inlineStr">
         <is>
           <t>University of North Carolina at Chapel Hill, Gillings School of Global Public Health, Department of Environmental Science &amp; Engineering, 135 Dauer Drive, Chapel Hill, NC 27599, United States of America</t>
+        </is>
+      </c>
+      <c r="O174" t="inlineStr">
+        <is>
+          <t>United States of America</t>
         </is>
       </c>
       <c r="W174" t="b">

</xml_diff>

<commit_message>
Rewrite expired supp_url and paper_url links to stable locations (#10)
343 washdev supp_url values were pre-signed Silverchair CDN links that
expired in January 2024, and 3 uncnewsletter paper_url values were Google
Scholar alert redirects. Both are now canonical: the Silverchair links
become https://doi.org/<doi> URLs (the DOI is recovered from the link
path), and the Scholar redirects are decoded to their target URLs. The
high-entropy Signature and scisig tokens that tripped secret scanners are
gone. No re-collection was needed.

Two reproducible helpers in data-raw/helpers.R do the rewrites:
canonicalize_silverchair_url() and decode_scholar_redirect(). Only
washdev$supp_url and uncnewsletter$paper_url changed; row counts and all
other columns are identical, and ploswater is untouched.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/inst/extdata/uncnewsletter.xlsx
+++ b/inst/extdata/uncnewsletter.xlsx
@@ -4832,7 +4832,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>https://scholar.google.com/scholar_url?url=https://ajph.aphapublications.org/doi/pdf/10.2105/AJPH.2022.307003%3Fdownload%3Dtrue&amp;hl=en&amp;sa=X&amp;d=3962241131938486649&amp;ei=H1Q7Y6aFPO2KywSS3bH4Bg&amp;scisig=AAGBfm3Q4X2sCbJJGTgTcSrsGU_FdUVJcw&amp;oi=scholaralrt&amp;hist=hZvSJggAAAAJ:7463423130094204642:AAGBfm306n8jEm7p9E06Y9mqflGSBiV6Pg&amp;html=&amp;pos=0&amp;folt=kw-top</t>
+          <t>https://ajph.aphapublications.org/doi/pdf/10.2105/AJPH.2022.307003?download=true</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -4910,7 +4910,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>https://scholar.google.com/scholar_url?url=https://pubs.acs.org/doi/full/10.1021/acsestwater.2c00157&amp;hl=en&amp;sa=X&amp;d=1709742523088559831&amp;ei=Dg_7YtkJhJjLBKCbvNAC&amp;scisig=AAGBfm0jov0_aWmZMwe4s6j4e9vubbdcbA&amp;oi=scholaralrt&amp;hist=hZvSJggAAAAJ:3226461804228696973:AAGBfm3ju-C3kL6mSiPesevK78XQ69Qd6A&amp;html=&amp;pos=2&amp;folt=kw</t>
+          <t>https://pubs.acs.org/doi/full/10.1021/acsestwater.2c00157</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -4993,7 +4993,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>https://scholar.google.com/scholar_url?url=https://onlinelibrary.wiley.com/doi/pdfdirect/10.1111/hir.12445&amp;hl=en&amp;sa=X&amp;d=7293212103073901469&amp;ei=2fm2YrzQKtHjmQGNwb84&amp;scisig=AAGBfm1zjx3-V2aCgS0L1xZx26MYDvF-tg&amp;oi=scholaralrt&amp;hist=hZvSJggAAAAJ:3552202248086981277:AAGBfm3xoOKMdpREzJ__fgBb7pdlMpLHFA&amp;html=&amp;pos=1&amp;folt=kw</t>
+          <t>https://onlinelibrary.wiley.com/doi/pdfdirect/10.1111/hir.12445</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">

</xml_diff>